<commit_message>
chore: atualiza planilha normativos_radar.xlsx
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$AC$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$J$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$AC$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$J$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC13"/>
+  <dimension ref="A1:AC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -865,22 +865,22 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Regulamenta o processo de autorização de funcionamento de instituições de pagamento e altera procedimentos de licenciamento no âmbito do Banco Central do Brasil.</t>
+          <t>Altera a Instrução Normativa BCB nº 693, de 19 de dezembro de 2025 que estabelece os procedimentos para a remessa ao Banco Central do Brasil de informações relativas a prestação de serviços de ativos virtuais no mercado de câmbio de que trata a Resolução BCB nº 521, de 10 de novembro de 2025.</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -905,7 +905,7 @@
         <v>2</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N3" s="5" t="n">
         <v>1</v>
@@ -917,7 +917,7 @@
         <v>2</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>Financiamento / Operações</t>
+          <t>Compliance Geral</t>
         </is>
       </c>
       <c r="T3" s="5" t="inlineStr">
@@ -936,12 +936,12 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>Pendente de avaliação</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>30 dias corridos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -956,27 +956,27 @@
       </c>
       <c r="Y3" s="5" t="inlineStr">
         <is>
-          <t>arranjos_pagamento</t>
+          <t>geral</t>
         </is>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
-          <t>pagamento, banco central</t>
+          <t>banco central</t>
         </is>
       </c>
       <c r="AA3" s="5" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=736</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AB3" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/instrucao_normativa_bcb_736.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AC3" s="5" t="inlineStr">
         <is>
-          <t>2026-05-22 15:41</t>
+          <t>2026-05-27 16:06</t>
         </is>
       </c>
     </row>
@@ -998,22 +998,22 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Estabelece procedimentos operacionais e prazos para o envio de informações regulatórias ao Banco Central do Brasil no âmbito do Sistema de Informações de Créditos (SCR).</t>
+          <t>Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Reguladas pelo Banco Central do Brasil(Cosif).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+          <t>Verificar</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>Crédito / Cartões, Tecnologia / Seg. Cibernética, Financiamento / Operações, Reporte Regulatório</t>
+          <t>Reporte Regulatório</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
@@ -1069,12 +1069,12 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>Pendente de avaliação</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>30 dias corridos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -1089,27 +1089,27 @@
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>credito</t>
+          <t>cosif</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>crédito, banco central</t>
+          <t>banco central, cosif</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/instrucao_normativa_bcb_737.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22 15:41</t>
+          <t>2026-05-27 16:06</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>Verificar</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Financiamento / Operações</t>
+          <t>Compliance Geral</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>Pendente de avaliação</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>30 dias corridos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_bcb_568.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22 15:41</t>
+          <t>2026-05-27 16:06</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Altera a Resolução BCB nº 343, de 4 de outubro de 2023, que dispõe sobre as medidas necessárias à execução do compartilhamento de dados e informações sobre indícios de fraudes.</t>
+          <t>Altera a Resolução BCB nº 343, de 4 de outubro de 2023, que dispõe sobre as medidas necessárias à execução do compartilhamento de dados e informações sobre indícios de fraudes de que trata a Resolução Conjunta nº 6, de 23 de maio de 2023.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1407,7 +1407,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>Verificar</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1434,7 +1434,7 @@
         <v>6</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>2</v>
@@ -1449,7 +1449,7 @@
         <v>2</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="S7" s="5" t="inlineStr">
         <is>
-          <t>PLD/FT e Prevenção a Fraudes, Reporte Regulatório</t>
+          <t>PLD/FT e Prevenção a Fraudes</t>
         </is>
       </c>
       <c r="T7" s="5" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="U7" s="5" t="inlineStr">
         <is>
-          <t>Pendente de avaliação</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>30 dias corridos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1498,17 +1498,17 @@
       </c>
       <c r="AA7" s="5" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=569</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AB7" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_bcb_569.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AC7" s="5" t="inlineStr">
         <is>
-          <t>2026-05-22 15:41</t>
+          <t>2026-05-27 16:06</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Altera a Resolução BCB nº 517, de 3 de novembro de 2025, que dispõe sobre os procedimentos a serem observados pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco Central.</t>
+          <t>Altera a Resolução BCB nº 517, de 3 de novembro de 2025, que dispõe sobre os procedimentos a serem observados pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco Central do Brasil na apuração do limite mínimo de capital social integralizado e de patrimônio líquido.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>Verificar</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Gestão Prudencial, Financiamento / Operações</t>
+          <t>Gestão Prudencial</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
@@ -1601,12 +1601,12 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>Pendente de avaliação</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
-          <t>30 dias corridos</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W8" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>arranjos_pagamento</t>
+          <t>geral</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -1631,17 +1631,17 @@
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=570</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_bcb_570.md</t>
+          <t>—</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-22 15:41</t>
+          <t>2026-05-27 16:06</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>resolucao_cmn_5304</t>
+          <t>resolucao_cmn_5305</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1924,22 +1924,22 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>5304</t>
+          <t>5305</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aquisição dos itens de que trata o art. 2º da Medida Provisória.</t>
+          <t>Altera as condições de abertura e manutenção de contas de depósitos e de poupança e a prestação de serviços por instituições financeiras, conforme regulamentação do Conselho Monetário Nacional.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>Financiamento / Operações</t>
+          <t>Compliance Geral</t>
         </is>
       </c>
       <c r="T11" s="5" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="Y11" s="5" t="inlineStr">
         <is>
-          <t>geral</t>
+          <t>arranjos_pagamento</t>
         </is>
       </c>
       <c r="Z11" s="5" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="AA11" s="5" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
         </is>
       </c>
       <c r="AB11" s="5" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_cmn_5304.md</t>
+          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_cmn_5305.md</t>
         </is>
       </c>
       <c r="AC11" s="5" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>resolucao_cmn_5305</t>
+          <t>resolucao_cmn_5306</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2057,12 +2057,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>5305</t>
+          <t>5306</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Altera as condições de abertura e manutenção de contas de depósitos e de poupança e a prestação de serviços por instituições financeiras, conforme regulamentação do Conselho Monetário Nacional.</t>
+          <t>Dispõe sobre limites operacionais, controles internos e a gestão de riscos aplicáveis às instituições financeiras autorizadas a funcionar pelo Banco Central do Brasil.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Compliance Geral</t>
+          <t>Financiamento / Operações</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
@@ -2153,22 +2153,22 @@
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>arranjos_pagamento</t>
+          <t>geral</t>
         </is>
       </c>
       <c r="Z12" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>banco central</t>
         </is>
       </c>
       <c r="AA12" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
         </is>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_cmn_5305.md</t>
+          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_cmn_5306.md</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
@@ -2177,141 +2177,8 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5306</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>5306</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Dispõe sobre limites operacionais, controles internos e a gestão de riscos aplicáveis às instituições financeiras autorizadas a funcionar pelo Banco Central do Brasil.</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-20</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>🟡</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="L13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q13" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="R13" s="5" t="inlineStr">
-        <is>
-          <t>Provável</t>
-        </is>
-      </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>Financiamento / Operações</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
-      <c r="V13" s="5" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="W13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="X13" s="5" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="Y13" s="5" t="inlineStr">
-        <is>
-          <t>geral</t>
-        </is>
-      </c>
-      <c r="Z13" s="5" t="inlineStr">
-        <is>
-          <t>banco central</t>
-        </is>
-      </c>
-      <c r="AA13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
-        </is>
-      </c>
-      <c r="AB13" s="5" t="inlineStr">
-        <is>
-          <t>https://github.com/giovannabatistutti-ctrl/normativos_md/blob/main/resolucao_cmn_5306.md</t>
-        </is>
-      </c>
-      <c r="AC13" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-22 15:41</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AC13"/>
+  <autoFilter ref="A1:AC12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2322,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -2382,11 +2249,11 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>73%</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -2405,11 +2272,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -2441,7 +2308,7 @@
         </is>
       </c>
       <c r="F5" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -2508,21 +2375,21 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>🔵 Pendente de avaliação</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="n">
         <v>6</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>🔵 Pendente de avaliação</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -2614,11 +2481,11 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Financiamento / Operações</t>
+          <t>Compliance Geral</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
@@ -2658,21 +2525,21 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>instrucao_normativa_bcb_736</t>
+          <t>resolucao_bcb_499</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>736</t>
+          <t>499</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
@@ -2698,21 +2565,21 @@
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>instrucao_normativa_bcb_737</t>
+          <t>resolucao_cmn_5</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
@@ -2738,21 +2605,21 @@
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>resolucao_bcb_499</t>
+          <t>resolucao_cmn_5303</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>499</t>
+          <t>5303</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
@@ -2774,25 +2641,25 @@
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>Pagamentos Pix</t>
+          <t>Financiamento / Operações</t>
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>resolucao_bcb_568</t>
+          <t>resolucao_cmn_5305</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
-          <t>568</t>
+          <t>5305</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -2814,7 +2681,7 @@
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>PLD/FT e Prevenção a Fraudes</t>
+          <t>Pagamentos Pix</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
@@ -2822,17 +2689,17 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>resolucao_bcb_569</t>
+          <t>resolucao_cmn_5306</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>569</t>
+          <t>5306</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
@@ -2854,209 +2721,21 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Gestão Prudencial</t>
+          <t>PLD/FT e Prevenção a Fraudes</t>
         </is>
       </c>
       <c r="B26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="10" t="inlineStr">
-        <is>
-          <t>resolucao_bcb_570</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>570</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Compliance Geral</t>
+          <t>Gestão Prudencial</t>
         </is>
       </c>
       <c r="B27" s="9" t="n">
         <v>1</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5303</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>5303</t>
-        </is>
-      </c>
-      <c r="G28" s="10" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="10" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5304</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>5304</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5305</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>5305</t>
-        </is>
-      </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5306</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>5306</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I31" s="9" t="inlineStr">
-        <is>
-          <t>Pendente de avaliação</t>
-        </is>
       </c>
     </row>
   </sheetData>
@@ -3078,7 +2757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -3194,7 +2873,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>1</v>
@@ -3206,7 +2885,7 @@
         <v>2</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -3331,7 +3010,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>2</v>
@@ -3346,7 +3025,7 @@
         <v>2</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
@@ -3457,7 +3136,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>resolucao_cmn_5304</t>
+          <t>resolucao_cmn_5305</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -3467,7 +3146,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>5304</t>
+          <t>5305</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
@@ -3492,7 +3171,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>resolucao_cmn_5305</t>
+          <t>resolucao_cmn_5306</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -3502,7 +3181,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>5305</t>
+          <t>5306</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
@@ -3524,43 +3203,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5306</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>5306</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>9</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I13"/>
+  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3571,7 +3215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3752,57 +3396,161 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>resolu__o_cmn_5</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aquisição dos itens de que trata o art. 3º da Medida Provisória nº 1.353, de 30 de abril de 2026.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo de atuação do iFood Pago</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-26 18:34</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
           <t>resolu__o_cmn_5001</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Resolução CMN</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>5001</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Dispõe sobre as condições para concessão de crédito rural para produtores agropecuários.</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>2026-01-15</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Tema fora do escopo de atuação do iFood Pago</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/normativos/detalhaormativo/5001</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I6" s="13" t="inlineStr">
         <is>
           <t>2026-05-22 18:28</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
     </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>resolucao_cmn_5304</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>5304</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aquisição dos itens de que trata o art. 2º da Medida Provisória.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo de atuação do iFood Pago</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibernormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-22 15:41</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:J5"/>
+  <autoFilter ref="A2:J7"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 01:52)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -673,11 +673,7 @@
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 735 — 2026-05-07</t>
@@ -688,21 +684,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -723,16 +707,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -755,11 +731,7 @@
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Resolução BCB nº 568 — 2026-05-07</t>
@@ -770,21 +742,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -805,16 +765,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O3" s="4" t="inlineStr"/>
+      <c r="P3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -837,11 +789,7 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5303 — 2026-05-14</t>
@@ -852,21 +800,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -887,16 +823,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5303</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -919,46 +847,18 @@
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 736 — 2026-05-16</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Regulamenta o processo de autorização de funcionamento de instituições de pagamento e altera procedimentos de licenciamento no âmbito do Banco Central do Brasil.</t>
@@ -969,16 +869,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Instrucao_Normativa_BCB/736</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1001,46 +893,18 @@
           <t>2026-05-19</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 737 — 2026-05-19</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Estabelece procedimentos operacionais e prazos para o envio de informações regulatórias ao Banco Central do Brasil no âmbito do Sistema de Informações de Créditos (SCR).</t>
@@ -1051,16 +915,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Instrucao_Normativa_BCB/737</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1083,11 +939,7 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 736 — 2026-05-20</t>
@@ -1098,21 +950,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1133,16 +973,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=736</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O7" s="4" t="inlineStr"/>
+      <c r="P7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1180,11 +1012,7 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr">
         <is>
           <t>MÉDIO</t>
@@ -1202,7 +1030,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Altera dispositivos normativos existentes. Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1215,16 +1043,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -1247,11 +1067,7 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 736 — 2026-05-20</t>
@@ -1262,21 +1078,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1297,16 +1101,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=736</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O9" s="4" t="inlineStr"/>
+      <c r="P9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1329,11 +1125,7 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 737 — 2026-05-20</t>
@@ -1344,21 +1136,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1379,16 +1159,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1411,46 +1183,18 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Resolução BCB nº 499 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
       <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Dispõe sobre a abertura, manutenção e movimentação de contas de pagamento pré-pagas e sobre o serviço de pagamento instantâneo no âmbito do ecossistema Pix, alterando a Resolução BCB nº 1, de 2020.</t>
@@ -1461,16 +1205,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_BCB/499</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1493,46 +1229,18 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5305 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Altera as condições de abertura e manutenção de contas de depósitos e de poupança e a prestação de serviços por instituições financeiras, conforme regulamentação do Conselho Monetário Nacional.</t>
@@ -1543,16 +1251,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_CMN/5305</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O12" s="2" t="inlineStr"/>
+      <c r="P12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1575,46 +1275,18 @@
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5306 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Dispõe sobre limites operacionais, controles internos e a gestão de riscos aplicáveis às instituições financeiras autorizadas a funcionar pelo Banco Central do Brasil.</t>
@@ -1625,16 +1297,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_CMN/5306</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1657,11 +1321,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Resolução BCB nº 569 — 2026-05-21</t>
@@ -1672,21 +1332,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1707,16 +1355,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=569</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1739,11 +1379,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Resolução BCB nº 570 — 2026-05-21</t>
@@ -1754,21 +1390,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1789,16 +1413,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=570</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O15" s="4" t="inlineStr"/>
+      <c r="P15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1821,11 +1437,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5 — 2026-05-21</t>
@@ -1836,21 +1448,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1871,16 +1471,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O16" s="2" t="inlineStr"/>
+      <c r="P16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1903,11 +1495,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5 — 2026-05-21</t>
@@ -1918,21 +1506,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -1953,16 +1529,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1985,11 +1553,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Resolução BCB nº 570 — 2026-05-21</t>
@@ -2000,21 +1564,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -2035,16 +1587,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=570</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O18" s="2" t="inlineStr"/>
+      <c r="P18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -2067,11 +1611,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5304 — 2026-05-21</t>
@@ -2082,21 +1622,9 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
       <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -2117,16 +1645,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2149,11 +1669,7 @@
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5305 — 2026-05-21</t>
@@ -2164,21 +1680,9 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -2199,16 +1703,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O20" s="2" t="inlineStr"/>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -2231,11 +1727,7 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E21" s="4" t="inlineStr"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5 — 2026-05-22</t>
@@ -2246,21 +1738,9 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -2281,16 +1761,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O21" s="4" t="inlineStr"/>
+      <c r="P21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2313,11 +1785,7 @@
           <t>2026-05-22</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Resolução CMN nº 5306 — 2026-05-22</t>
@@ -2328,21 +1796,9 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -2363,16 +1819,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O22" s="2" t="inlineStr"/>
+      <c r="P22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -2554,11 +2002,7 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="5" t="inlineStr">
         <is>
           <t>MÉDIO</t>
@@ -2576,7 +2020,7 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Altera dispositivos normativos existentes. Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
@@ -2589,16 +2033,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P25" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O25" s="4" t="inlineStr"/>
+      <c r="P25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2636,11 +2072,7 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="5" t="inlineStr">
         <is>
           <t>MÉDIO</t>
@@ -2658,7 +2090,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Altera dispositivos normativos existentes. Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2671,16 +2103,8 @@
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+      <c r="P26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -2688,81 +2112,25 @@
           <t>bc_-_instrução_normativa_bcb_n_735_de_06052026</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr"/>
+      <c r="O27" s="4" t="inlineStr"/>
+      <c r="P27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2770,81 +2138,25 @@
           <t>bc_-_resolução_bcb_n_568_de_06052026</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
+      <c r="P28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -2939,7 +2251,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52914</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -2947,7 +2259,11 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr"/>
@@ -2965,7 +2281,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -2973,7 +2289,11 @@
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr"/>
@@ -2991,167 +2311,55 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
       <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=738</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52910</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="4" t="inlineStr"/>
-      <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="P35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52914</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52906</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr"/>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="P37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52915</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=738</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P38"/>
+  <autoFilter ref="A1:P34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3162,7 +2370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3224,7 +2432,7 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -3247,7 +2455,7 @@
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -3270,7 +2478,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -3370,7 +2578,7 @@
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C13" s="11" t="n">
         <v>0</v>
@@ -3395,12 +2603,6 @@
       </c>
       <c r="G14" s="12" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="F15" s="11" t="inlineStr"/>
-      <c r="G15" s="11" t="n">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3420,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3520,41 +2722,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -3582,41 +2756,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -3644,41 +2790,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -3701,51 +2819,15 @@
           <t>Instrução Normativa BCB nº 736 — 2026-05-16</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -3763,51 +2845,15 @@
           <t>Instrução Normativa BCB nº 737 — 2026-05-19</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -3830,41 +2876,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -3892,30 +2910,20 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="E8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -3954,41 +2962,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4016,41 +2996,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4073,51 +3025,15 @@
           <t>Resolução BCB nº 499 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -4135,51 +3051,15 @@
           <t>Resolução CMN nº 5305 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -4197,51 +3077,15 @@
           <t>Resolução CMN nº 5306 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -4264,41 +3108,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4326,41 +3142,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4388,41 +3176,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4450,41 +3210,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4512,41 +3244,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4574,41 +3278,13 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4636,41 +3312,13 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4698,41 +3346,13 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4760,41 +3380,13 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Vigência imediata</t>
@@ -4914,30 +3506,20 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="E25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
@@ -4976,30 +3558,20 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="E26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
@@ -5018,187 +3590,43 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L32"/>
+  <autoFilter ref="A1:L28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 01:57)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -48,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +73,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF8800"/>
       </patternFill>
     </fill>
     <fill>
@@ -137,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -163,10 +168,13 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -178,10 +186,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -853,9 +861,17 @@
           <t>Instrução Normativa BCB nº 736 — 2026-05-16</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
@@ -1013,7 +1029,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -1189,9 +1205,17 @@
           <t>Resolução BCB nº 499 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr"/>
-      <c r="I11" s="4" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
@@ -1617,7 +1641,7 @@
           <t>Resolução CMN nº 5304 — 2026-05-21</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1675,7 +1699,7 @@
           <t>Resolução CMN nº 5305 — 2026-05-21</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1791,7 +1815,7 @@
           <t>Resolução CMN nº 5306 — 2026-05-22</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1849,7 +1873,7 @@
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1859,7 +1883,7 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
@@ -1921,7 +1945,7 @@
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1931,7 +1955,7 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
@@ -2003,7 +2027,7 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -2073,7 +2097,7 @@
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -2169,7 +2193,7 @@
       <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2199,7 +2223,7 @@
       <c r="D30" s="2" t="inlineStr"/>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2229,7 +2253,7 @@
       <c r="D31" s="4" t="inlineStr"/>
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="8" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2259,7 +2283,7 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="8" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2289,7 +2313,7 @@
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="8" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2335,7 +2359,7 @@
           <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
         </is>
       </c>
-      <c r="G34" s="8" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
@@ -2383,120 +2407,120 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>📊 Por Classificação</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>🚨 Por Criticidade</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Classificação</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Criticidade</t>
         </is>
       </c>
-      <c r="F2" s="10" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>✅ Aplicável</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="C3" s="11" t="inlineStr">
-        <is>
-          <t>45%</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="inlineStr">
+      <c r="B3" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>52%</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>🔴 Crítico</t>
         </is>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>⚠️ Monitorar</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>🟠 Alto</t>
         </is>
       </c>
-      <c r="F4" s="12" t="n">
-        <v>0</v>
+      <c r="F4" s="13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>❌ Não Aplicável</t>
         </is>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="12" t="inlineStr">
         <is>
           <t>18%</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>🟡 Médio</t>
         </is>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="12" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>🟢 Baixo</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F6" s="13" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2504,104 +2528,104 @@
     <row r="8"/>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>📅 Por Mês</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>🎯 Por Confiança</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Mês</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Aplicável</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Monitorar</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>Confiança</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>May/2026</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>26</v>
       </c>
-      <c r="C12" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="D12" s="12" t="n">
+      <c r="C12" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="D12" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="12" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="14">
-      <c r="F14" s="12" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>BAIXA</t>
         </is>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2819,14 +2843,22 @@
           <t>Instrução Normativa BCB nº 736 — 2026-05-16</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
       <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
@@ -3025,14 +3057,22 @@
           <t>Resolução BCB nº 499 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
       <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr"/>
       <c r="J11" s="4" t="inlineStr"/>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="L11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
@@ -3651,49 +3691,49 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>ℹ️  Backlog de normativos classificados como Não Aplicáveis ao iFood Pago. Use para consulta e revisão periódica.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>Número</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="15" t="inlineStr">
         <is>
           <t>Data Publicação</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="15" t="inlineStr">
         <is>
           <t>Título</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>Justificativa (Por que não se aplica)</t>
         </is>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>Confiança</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
+      <c r="H2" s="15" t="inlineStr">
         <is>
           <t>Data Análise</t>
         </is>
@@ -3722,22 +3762,22 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>normativos_52911</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr"/>
-      <c r="C4" s="15" t="inlineStr"/>
-      <c r="D4" s="15" t="inlineStr"/>
-      <c r="E4" s="15" t="inlineStr"/>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr"/>
+      <c r="C4" s="16" t="inlineStr"/>
+      <c r="D4" s="16" t="inlineStr"/>
+      <c r="E4" s="16" t="inlineStr"/>
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr"/>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>2026-05-27</t>
         </is>
@@ -3766,22 +3806,22 @@
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>normativos_52914</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr"/>
-      <c r="C6" s="15" t="inlineStr"/>
-      <c r="D6" s="15" t="inlineStr"/>
-      <c r="E6" s="15" t="inlineStr"/>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr"/>
+      <c r="C6" s="16" t="inlineStr"/>
+      <c r="D6" s="16" t="inlineStr"/>
+      <c r="E6" s="16" t="inlineStr"/>
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr"/>
-      <c r="H6" s="15" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr"/>
+      <c r="H6" s="16" t="inlineStr">
         <is>
           <t>2026-05-27</t>
         </is>
@@ -3810,42 +3850,42 @@
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>normativos_52915</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>738</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
         </is>
       </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:H8"/>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 02:00)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -82,17 +82,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
     <fill>
@@ -915,9 +915,17 @@
           <t>Instrução Normativa BCB nº 737 — 2026-05-19</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
@@ -1029,7 +1037,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -1641,7 +1649,7 @@
           <t>Resolução CMN nº 5304 — 2026-05-21</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1699,7 +1707,7 @@
           <t>Resolução CMN nº 5305 — 2026-05-21</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1815,7 +1823,7 @@
           <t>Resolução CMN nº 5306 — 2026-05-22</t>
         </is>
       </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1873,7 +1881,7 @@
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1883,7 +1891,7 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
@@ -1945,7 +1953,7 @@
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>MONITORAR</t>
         </is>
@@ -1955,7 +1963,7 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
@@ -2027,7 +2035,7 @@
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -2097,7 +2105,7 @@
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>MÉDIO</t>
         </is>
@@ -2136,23 +2144,63 @@
           <t>bc_-_instrução_normativa_bcb_n_735_de_06052026</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>735</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-      <c r="I27" s="4" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>A norma aborda temas relevantes ao iFood Pago (crédito) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>Altera o leiaute, as instruções de preenchimento e as instruções de programas públicos do documento de código 3040 - Dados de Risco de Crédito, do Sistema de Informações de Créditos (SCR), de que trat</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735</t>
+        </is>
+      </c>
       <c r="O27" s="4" t="inlineStr"/>
       <c r="P27" s="4" t="inlineStr"/>
     </row>
@@ -2162,23 +2210,63 @@
           <t>bc_-_resolução_bcb_n_568_de_06052026</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>568</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr"/>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>A norma aborda temas relevantes ao iFood Pago (banco central) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
+        </is>
+      </c>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
     </row>
@@ -2475,11 +2563,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -2521,7 +2609,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7"/>
@@ -2578,13 +2666,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>17</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -2602,7 +2690,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>0</v>
@@ -2616,7 +2704,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -2877,14 +2965,22 @@
           <t>Instrução Normativa BCB nº 737 — 2026-05-19</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
@@ -3630,39 +3726,71 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>735</t>
+        </is>
+      </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="E27" s="4" t="inlineStr"/>
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="4" t="inlineStr"/>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr"/>
       <c r="J27" s="4" t="inlineStr"/>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>568</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 02:02)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -1267,7 +1267,11 @@
           <t>Resolução CMN nº 5305 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
@@ -1313,7 +1317,11 @@
           <t>Resolução CMN nº 5306 — 2026-05-20</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr"/>
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr"/>
@@ -2563,11 +2571,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -2672,7 +2680,7 @@
         <v>17</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -3187,7 +3195,11 @@
           <t>Resolução CMN nº 5305 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
@@ -3213,7 +3225,11 @@
           <t>Resolução CMN nº 5306 — 2026-05-20</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 19:53)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normativos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilares" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Normativos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pilares" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -557,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1657,9 +1659,9 @@
           <t>Resolução CMN nº 5304 — 2026-05-21</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
@@ -2303,7 +2305,7 @@
       <c r="N29" s="4" t="inlineStr"/>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P29" s="4" t="inlineStr"/>
@@ -2333,7 +2335,7 @@
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr"/>
@@ -2363,7 +2365,7 @@
       <c r="N31" s="4" t="inlineStr"/>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P31" s="4" t="inlineStr"/>
@@ -2371,7 +2373,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -2379,9 +2381,9 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2393,7 +2395,7 @@
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr"/>
@@ -2401,7 +2403,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -2409,9 +2411,9 @@
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -2423,7 +2425,7 @@
       <c r="N33" s="4" t="inlineStr"/>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="P33" s="4" t="inlineStr"/>
@@ -2431,55 +2433,155 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
+          <t>normativos_52907</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=738</t>
-        </is>
-      </c>
-      <c r="O34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="P34" s="2" t="inlineStr"/>
     </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52910</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+      <c r="M35" s="4" t="inlineStr"/>
+      <c r="N35" s="4" t="inlineStr"/>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52914</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr"/>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P34"/>
+  <autoFilter ref="A1:P38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2548,11 +2650,11 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -2571,11 +2673,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -2594,11 +2696,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2674,13 +2776,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>17</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -2698,10 +2800,10 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>0</v>
@@ -2712,7 +2814,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -2742,7 +2844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3417,12 +3519,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>5304</t>
+          <t>5305</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5304 — 2026-05-21</t>
+          <t>Resolução CMN nº 5305 — 2026-05-21</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -3451,17 +3553,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>5305</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5305 — 2026-05-21</t>
+          <t>Resolução CMN nº 5 — 2026-05-22</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -3485,17 +3587,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>5306</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5 — 2026-05-22</t>
+          <t>Resolução CMN nº 5306 — 2026-05-22</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -3514,17 +3616,17 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>5306</t>
+          <t>735</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5306 — 2026-05-22</t>
+          <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -3532,33 +3634,45 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Vigência imediata</t>
-        </is>
-      </c>
+      <c r="E22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>568</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
+          <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -3604,53 +3718,59 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
+          <t>Resolução BCB nº 568 — 2026-05-07</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>6 — Quadrante K</t>
+        </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr"/>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>30 dias corridos</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>568</t>
+          <t>737</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB nº 568 — 2026-05-07</t>
+          <t>Instrução Normativa BCB nº 737 — 2026-05-25</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -3697,64 +3817,46 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>735</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB nº 737 — 2026-05-25</t>
+          <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>6 — Quadrante K</t>
-        </is>
-      </c>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>30 dias corridos</t>
-        </is>
-      </c>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>735</t>
+          <t>568</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 735 de 06/05/2026</t>
+          <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -3776,24 +3878,12 @@
       <c r="L27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>568</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 568 de 06/05/2026</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
@@ -3802,15 +3892,65 @@
       <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="K28" s="2" t="inlineStr"/>
       <c r="L28" s="2" t="inlineStr"/>
     </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="4" t="inlineStr"/>
+      <c r="C29" s="4" t="inlineStr"/>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="4" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L28"/>
+  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3821,15 +3961,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
@@ -3886,29 +4026,41 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr"/>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr"/>
+          <t>2026-05-21_resolucao_cmn_5304</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>5304</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN nº 5304 — 2026-05-21</t>
+        </is>
+      </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Tema fora do escopo do iFood Pago</t>
+          <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
+      <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr"/>
@@ -3923,14 +4075,14 @@
       <c r="G4" s="16" t="inlineStr"/>
       <c r="H4" s="16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr"/>
@@ -3945,14 +4097,14 @@
       <c r="G5" s="4" t="inlineStr"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr"/>
@@ -3967,14 +4119,14 @@
       <c r="G6" s="16" t="inlineStr"/>
       <c r="H6" s="16" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52914</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
@@ -3989,53 +4141,254 @@
       <c r="G7" s="4" t="inlineStr"/>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr"/>
+      <c r="C8" s="16" t="inlineStr"/>
+      <c r="D8" s="16" t="inlineStr"/>
+      <c r="E8" s="16" t="inlineStr"/>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>normativos_52915</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H8"/>
+  <autoFilter ref="A2:H9"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Número</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Título</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Classificação</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Confiança (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SLA (min)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Avaliação Tipo</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Risco</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Data Análise</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Feedback ID</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Feedback Autor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52913_test</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN nº 5306 - Teste de auditoria</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>CRÍTICO</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52913_test</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>5306</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN nº 5306 - Teste de auditoria</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>feedback_1</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 21:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Normativos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Pilares" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normativos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilares" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog NÃO APLICÁVEL" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -50,7 +50,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +117,11 @@
         <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -144,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -194,6 +199,7 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -571,7 +577,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
@@ -2283,67 +2289,145 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="4" t="inlineStr"/>
+          <t>normativos_52914</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P29" s="4" t="inlineStr"/>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>agregador</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr"/>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr"/>
@@ -2373,7 +2457,7 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -2381,9 +2465,9 @@
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -2403,7 +2487,7 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -2411,9 +2495,9 @@
       <c r="D33" s="4" t="inlineStr"/>
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -2433,7 +2517,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
@@ -2463,7 +2547,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -2493,7 +2577,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
@@ -2501,9 +2585,9 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2523,7 +2607,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -2531,9 +2615,9 @@
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -2553,7 +2637,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
@@ -2580,8 +2664,58 @@
       </c>
       <c r="P38" s="2" t="inlineStr"/>
     </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
+      <c r="M39" s="4" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=738</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P38"/>
+  <autoFilter ref="A1:P39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2654,7 +2788,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -2673,11 +2807,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -2696,11 +2830,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2709,7 +2843,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -2776,13 +2910,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>17</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -2800,7 +2934,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>4</v>
@@ -2814,7 +2948,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -2844,7 +2978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2856,7 +2990,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
   </cols>
@@ -3878,30 +4012,68 @@
       <c r="L27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr"/>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="n">
+        <v>2.111111111111111</v>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr"/>
-      <c r="C29" s="4" t="inlineStr"/>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
@@ -3910,7 +4082,11 @@
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr"/>
       <c r="J29" s="4" t="inlineStr"/>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
@@ -3949,8 +4125,44 @@
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
     </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="4" t="inlineStr"/>
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L31"/>
+  <autoFilter ref="A1:L33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3961,14 +4173,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -4126,7 +4338,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr"/>
@@ -4148,49 +4360,43 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr"/>
-      <c r="C8" s="16" t="inlineStr"/>
-      <c r="D8" s="16" t="inlineStr"/>
-      <c r="E8" s="16" t="inlineStr"/>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr"/>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52915</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Tema fora do escopo do iFood Pago</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:H9"/>
+  <autoFilter ref="A2:H8"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -4204,16 +4410,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -4387,8 +4593,146 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>326.95</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>329.05</v>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52914</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>329.0833333333333</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 21:03)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -149,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,6 +200,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4410,7 +4411,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -4423,7 +4424,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -4731,8 +4732,66 @@
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
     </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB N° 738 de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>feedback_e2e_test_001</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 21:48)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2671,48 +2671,28 @@
           <t>normativos_52915</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
-        </is>
-      </c>
+      <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
+      <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr"/>
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=738</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr"/>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="P39" s="4" t="inlineStr"/>
     </row>
   </sheetData>
@@ -2911,7 +2891,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>17</v>
@@ -2935,7 +2915,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>4</v>
@@ -2949,7 +2929,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -4178,10 +4158,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -4364,37 +4344,21 @@
           <t>normativos_52915</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="E8" s="16" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
-        </is>
-      </c>
+      <c r="B8" s="16" t="inlineStr"/>
+      <c r="C8" s="16" t="inlineStr"/>
+      <c r="D8" s="16" t="inlineStr"/>
+      <c r="E8" s="16" t="inlineStr"/>
       <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Tema fora do escopo do iFood Pago</t>
         </is>
       </c>
-      <c r="G8" s="16" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr"/>
+      <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:H8"/>
@@ -4411,10 +4375,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -4790,8 +4754,104 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>instrucao_normativa_bcb_722</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instrução Normativa BCB nº 722, de 13 de abril de </t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>resolucao_conjunta_18_2025</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 202</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>60</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:L9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 21:49)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
   </definedNames>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P39"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2290,79 +2290,69 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>instrucao_normativa_bcb_722</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>722</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+          <t>Instrução Normativa BCB nº 722, de 13 de abril de 2026</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="n">
-        <v>2.111111111111111</v>
-      </c>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
-        </is>
-      </c>
+      <c r="L29" s="4" t="inlineStr"/>
       <c r="M29" s="4" t="inlineStr">
         <is>
-          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+          <t>Divulga a versão 8.2 do Manual Operacional do Diretório de Identificadores de Contas Transacionais (DICT), que compõe o Regulamento do Pix.</t>
         </is>
       </c>
       <c r="N29" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
-        </is>
-      </c>
-      <c r="O29" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+          <t>https://in.gov.br/web/dou/-/instrucao-normativa-bcb-n-722-de-13-de-abril-2026-699855491</t>
+        </is>
+      </c>
+      <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="4" t="inlineStr">
         <is>
-          <t>agregador</t>
+          <t>dou_html</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
+          <t>normativos_52914</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2380,11 +2370,7 @@
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+      <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
@@ -2405,7 +2391,9 @@
           <t>MÉDIO</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
@@ -2419,76 +2407,152 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
-        </is>
-      </c>
-      <c r="O30" s="2" t="inlineStr"/>
-      <c r="P30" s="2" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>agregador</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
+          <t>resolucao_conjunta_18_2025</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
       <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="P31" s="4" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>Dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco C</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr"/>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>dou_html</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr"/>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr"/>
@@ -2518,7 +2582,7 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
@@ -2526,9 +2590,9 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -2548,7 +2612,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -2556,9 +2620,9 @@
       <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
@@ -2578,7 +2642,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
@@ -2608,7 +2672,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -2638,7 +2702,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
@@ -2646,9 +2710,9 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2668,7 +2732,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -2676,9 +2740,9 @@
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -2695,8 +2759,68 @@
       </c>
       <c r="P39" s="4" t="inlineStr"/>
     </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
+      <c r="M41" s="4" t="inlineStr"/>
+      <c r="N41" s="4" t="inlineStr"/>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="P41" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P39"/>
+  <autoFilter ref="A1:P41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2707,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2765,11 +2889,11 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -2792,7 +2916,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -2801,7 +2925,7 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -2815,7 +2939,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -2887,17 +3011,17 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>May/2026</t>
+          <t>Apr/2026</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -2905,23 +3029,23 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>May/2026</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
@@ -2933,12 +3057,42 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Nov/2025</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
           <t>BAIXA</t>
         </is>
       </c>
       <c r="G14" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2959,7 +3113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3995,43 +4149,33 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>722</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+          <t>Instrução Normativa BCB nº 722, de 13 de abril de 2026</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>3</v>
-      </c>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="n">
-        <v>2.111111111111111</v>
-      </c>
+      <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr"/>
@@ -4057,12 +4201,22 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>3</v>
+      </c>
       <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
           <t>MÉDIO</t>
@@ -4071,9 +4225,21 @@
       <c r="L29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+        </is>
+      </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
@@ -4085,16 +4251,32 @@
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
       <c r="L30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
@@ -4103,7 +4285,11 @@
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr"/>
-      <c r="K31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
@@ -4142,8 +4328,44 @@
       <c r="K33" s="4" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr"/>
     </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr"/>
+      <c r="C35" s="4" t="inlineStr"/>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L33"/>
+  <autoFilter ref="A1:L35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 22:08)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$P$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -583,8 +583,9 @@
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="50" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -650,20 +651,25 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Racional de Risco</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Ementa</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Link BCB</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Data Análise</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Fonte Texto</t>
         </is>
@@ -714,18 +720,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Altera o leiaute, as instruções de preenchimento e as instruções de programas públicos do documento de código 3040 - Dados de Risco de Crédito, do Sistema de Informações de Créditos (SCR), de que trat</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -772,18 +779,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr"/>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr"/>
       <c r="P3" s="4" t="inlineStr"/>
+      <c r="Q3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -830,18 +838,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Altera normas da Seção 9 (Impedimentos Sociais, Ambientais e Climáticos) do Capítulo 2 (Condições Básicas) do Manual de Crédito Rural – MCR.</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5303</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -884,18 +893,19 @@
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Regulamenta o processo de autorização de funcionamento de instituições de pagamento e altera procedimentos de licenciamento no âmbito do Banco Central do Brasil.</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Instrucao_Normativa_BCB/736</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr"/>
       <c r="P5" s="4" t="inlineStr"/>
+      <c r="Q5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -938,18 +948,19 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Estabelece procedimentos operacionais e prazos para o envio de informações regulatórias ao Banco Central do Brasil no âmbito do Sistema de Informações de Créditos (SCR).</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Instrucao_Normativa_BCB/737</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -996,18 +1007,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Altera a Instrução Normativa BCB nº 693, de 19 de dezembro de 2025 que estabelece os procedimentos para a remessa ao Banco Central do Brasil de informações relativas a prestação de serviços de ativos </t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=736</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr"/>
       <c r="P7" s="4" t="inlineStr"/>
+      <c r="Q7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1066,18 +1078,19 @@
           <t>Altera dispositivos normativos existentes. Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Regu</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -1124,18 +1137,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Altera a Instrução Normativa BCB nº 693, de 19 de dezembro de 2025 que estabelece os procedimentos para a remessa ao Banco Central do Brasil de informações relativas a prestação de serviços de ativos </t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=736</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr"/>
       <c r="P9" s="4" t="inlineStr"/>
+      <c r="Q9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1182,18 +1196,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Regu</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1236,18 +1251,19 @@
       <c r="J11" s="4" t="inlineStr"/>
       <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="4" t="inlineStr"/>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Dispõe sobre a abertura, manutenção e movimentação de contas de pagamento pré-pagas e sobre o serviço de pagamento instantâneo no âmbito do ecossistema Pix, alterando a Resolução BCB nº 1, de 2020.</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="O11" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_BCB/499</t>
         </is>
       </c>
-      <c r="O11" s="4" t="inlineStr"/>
       <c r="P11" s="4" t="inlineStr"/>
+      <c r="Q11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1286,18 +1302,19 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Altera as condições de abertura e manutenção de contas de depósitos e de poupança e a prestação de serviços por instituições financeiras, conforme regulamentação do Conselho Monetário Nacional.</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_CMN/5305</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1336,18 +1353,19 @@
       <c r="J13" s="4" t="inlineStr"/>
       <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr"/>
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Dispõe sobre limites operacionais, controles internos e a gestão de riscos aplicáveis às instituições financeiras autorizadas a funcionar pelo Banco Central do Brasil.</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="O13" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo/Resolucao_CMN/5306</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr"/>
       <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1394,18 +1412,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Altera a Resolução BCB nº 343, de 4 de outubro de 2023, que dispõe sobre as medidas necessárias à execução do compartilhamento de dados e informações sobre indícios de fraudes de que trata a Resolução</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="O14" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=569</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr"/>
       <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1452,18 +1471,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Altera a Resolução BCB nº 517, de 3 de novembro de 2025, que dispõe sobre os procedimentos a serem observados pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco Ce</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="O15" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=570</t>
         </is>
       </c>
-      <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr"/>
+      <c r="Q15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1510,18 +1530,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aquisição dos itens de que trata o art. 2º da Medida Provisór</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -1568,18 +1589,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Estabelece as condições para a concessão de financiamentos destinados a capital de giro a prestadores de serviços aéreos regulares, na forma do art. 21 da Medida Provisória nº 1.349, de 7 de abril de </t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="O17" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
         </is>
       </c>
-      <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
+      <c r="Q17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1626,18 +1648,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Altera a Resolução BCB nº 517, de 3 de novembro de 2025, que dispõe sobre os procedimentos a serem observados pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco Ce</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=570</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -1684,18 +1707,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aquisição dos itens de que trata o art. 2º da Medida Provisór</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="O19" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5304</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr"/>
       <c r="P19" s="4" t="inlineStr"/>
+      <c r="Q19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -1742,18 +1766,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Estabelece as condições para a concessão de financiamentos destinados a capital de giro a prestadores de serviços aéreos regulares, na forma do art. 21 da Medida Provisória nº 1.349, de 7 de abril de </t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5305</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -1800,18 +1825,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="M21" s="4" t="inlineStr"/>
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Altera o art. 2º da Resolução CMN nº 5.097, de 24 de agosto de 2023, que define os critérios de elegibilidade para as operações de financiamento à inovação e à digitalização com recursos do Fundo de A</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="O21" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
         </is>
       </c>
-      <c r="O21" s="4" t="inlineStr"/>
       <c r="P21" s="4" t="inlineStr"/>
+      <c r="Q21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -1858,18 +1884,19 @@
           <t>Revisar com equipe de Compliance e verificar adequação operacional.</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Altera o art. 2º da Resolução CMN nº 5.097, de 24 de agosto de 2023, que define os critérios de elegibilidade para as operações de financiamento à inovação e à digitalização com recursos do Fundo de A</t>
         </is>
       </c>
-      <c r="N22" s="2" t="inlineStr">
+      <c r="O22" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5306</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1922,22 +1949,23 @@
           <t>A norma aborda temas relevantes ao iFood Pago (crédito) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Altera o leiaute, as instruções de preenchimento e as instruções de programas públicos do documento de código 3040 - Dados de Risco de Crédito, do Sistema de Informações de Créditos (SCR), de que trat</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="O23" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735</t>
         </is>
       </c>
-      <c r="O23" s="4" t="inlineStr">
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="Q23" s="4" t="inlineStr">
         <is>
           <t>html</t>
         </is>
@@ -1994,22 +2022,23 @@
           <t>A norma aborda temas relevantes ao iFood Pago (banco central) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
-      <c r="N24" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t>2026-05-26</t>
         </is>
       </c>
-      <c r="P24" s="2" t="inlineStr">
+      <c r="Q24" s="2" t="inlineStr">
         <is>
           <t>html</t>
         </is>
@@ -2072,18 +2101,19 @@
           <t>Altera dispositivos normativos existentes. Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="4" t="inlineStr"/>
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="O25" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O25" s="4" t="inlineStr"/>
       <c r="P25" s="4" t="inlineStr"/>
+      <c r="Q25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2142,18 +2172,19 @@
           <t>Altera dispositivos normativos existentes. Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>Altera as Instruções Normativas BCB ns. 426, 428, 429, 430, 431, 432 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Regu</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=737</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -2208,18 +2239,19 @@
           <t>A norma aborda temas relevantes ao iFood Pago (crédito) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr">
+      <c r="M27" s="4" t="inlineStr"/>
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Altera o leiaute, as instruções de preenchimento e as instruções de programas públicos do documento de código 3040 - Dados de Risco de Crédito, do Sistema de Informações de Créditos (SCR), de que trat</t>
         </is>
       </c>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="O27" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=735</t>
         </is>
       </c>
-      <c r="O27" s="4" t="inlineStr"/>
       <c r="P27" s="4" t="inlineStr"/>
+      <c r="Q27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2274,18 +2306,19 @@
           <t>A norma aborda temas relevantes ao iFood Pago (banco central) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
         </is>
       </c>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=568</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
+      <c r="Q28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -2308,7 +2341,11 @@
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>11 de maio de 2026.</t>
+        </is>
+      </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB nº 722, de 13 de abril de 2026</t>
@@ -2321,7 +2358,7 @@
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -2331,19 +2368,46 @@
       </c>
       <c r="J29" s="4" t="inlineStr"/>
       <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>🔴 APLICÁVEL — Instrução Normativa BCB nº 722/2026
+**1. Identificação**
+Foi publicada a Instrução Normativa BCB nº 722, de 13 de abril de 2026, que divulga a versão 8.2 do Manual Operacional do Diretório de Identificadores de Contas Transacionais (DICT), parte integrante do Regulamento do Pix. Revog
+### Avaliação de Risco:
+| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Alterações no Manual Operacional do DICT exigem revisão de fluxos e sistemas. |
+| ⚖️ Regulatório | 3 | Conformidade obrigatória com o Regulamento do Pix e o Manual Operacional do DICT. |
+| 💰 Financeiro | 2 | Potencial impacto financeiro limitado a ajustes operacionais. |
+| 👥 Clientes | 2 | Impacto indireto em clientes, relacionado à continuidade e segurança das operações Pix. |</t>
+        </is>
+      </c>
       <c r="M29" s="4" t="inlineStr">
         <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Alterações no Manual Operacional do DICT exigem revisão de fluxos e sistemas. |
+| ⚖️ Regulatório | 3 | Conformidade obrigatória com o Regulamento do Pix e o Manual Operacional do DICT. |
+| 💰 Financeiro | 2 | Potencial impacto financeiro limitado a ajustes operacionais. |
+| 👥 Clientes | 2 | Impacto indireto em clientes, relacionado à continuidade e segurança das operações Pix. |</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
           <t>Divulga a versão 8.2 do Manual Operacional do Diretório de Identificadores de Contas Transacionais (DICT), que compõe o Regulamento do Pix.</t>
         </is>
       </c>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="O29" s="4" t="inlineStr">
         <is>
           <t>https://in.gov.br/web/dou/-/instrucao-normativa-bcb-n-722-de-13-de-abril-2026-699855491</t>
         </is>
       </c>
-      <c r="O29" s="4" t="inlineStr"/>
       <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>dou_html</t>
         </is>
@@ -2400,22 +2464,23 @@
           <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
         </is>
       </c>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P30" s="2" t="inlineStr">
+      <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>agregador</t>
         </is>
@@ -2442,7 +2507,11 @@
           <t>2025-11-28</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>1º de janeiro de 2026.</t>
+        </is>
+      </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
@@ -2455,7 +2524,7 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
@@ -2465,19 +2534,46 @@
       </c>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>🔴 APLICÁVEL — Resolução Conjunta nº 18/2025
+**1. Identificação**
+Foi publicada a Resolução Conjunta nº 18, de 28 de novembro de 2025, que dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituiçõ
+### Avaliação de Risco:
+| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Exige ajustes em processos e sistemas de reporte para atender às novas exigências. |
+| ⚖️ Regulatório | 4 | Norma impõe obrigação direta ao iFood Pago, com risco de sanções em caso de não conformidade. |
+| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e controles, mas sem impacto direto em receitas. |
+| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
+        </is>
+      </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Exige ajustes em processos e sistemas de reporte para atender às novas exigências. |
+| ⚖️ Regulatório | 4 | Norma impõe obrigação direta ao iFood Pago, com risco de sanções em caso de não conformidade. |
+| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e controles, mas sem impacto direto em receitas. |
+| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
           <t>Dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco C</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="O31" s="4" t="inlineStr">
         <is>
           <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr"/>
       <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>dou_html</t>
         </is>
@@ -2536,18 +2632,19 @@
           <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -2572,12 +2669,13 @@
       <c r="L33" s="4" t="inlineStr"/>
       <c r="M33" s="4" t="inlineStr"/>
       <c r="N33" s="4" t="inlineStr"/>
-      <c r="O33" s="4" t="inlineStr">
+      <c r="O33" s="4" t="inlineStr"/>
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P33" s="4" t="inlineStr"/>
+      <c r="Q33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -2602,12 +2700,13 @@
       <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr"/>
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr"/>
+      <c r="Q34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -2632,12 +2731,13 @@
       <c r="L35" s="4" t="inlineStr"/>
       <c r="M35" s="4" t="inlineStr"/>
       <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr">
+      <c r="O35" s="4" t="inlineStr"/>
+      <c r="P35" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P35" s="4" t="inlineStr"/>
+      <c r="Q35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -2662,12 +2762,13 @@
       <c r="L36" s="2" t="inlineStr"/>
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr"/>
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P36" s="2" t="inlineStr"/>
+      <c r="Q36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -2692,12 +2793,13 @@
       <c r="L37" s="4" t="inlineStr"/>
       <c r="M37" s="4" t="inlineStr"/>
       <c r="N37" s="4" t="inlineStr"/>
-      <c r="O37" s="4" t="inlineStr">
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P37" s="4" t="inlineStr"/>
+      <c r="Q37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -2722,12 +2824,13 @@
       <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="inlineStr">
+      <c r="O38" s="2" t="inlineStr"/>
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -2752,12 +2855,13 @@
       <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
       <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr">
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P39" s="4" t="inlineStr"/>
+      <c r="Q39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -2782,12 +2886,13 @@
       <c r="L40" s="2" t="inlineStr"/>
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="inlineStr">
+      <c r="O40" s="2" t="inlineStr"/>
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P40" s="2" t="inlineStr"/>
+      <c r="Q40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -2812,15 +2917,16 @@
       <c r="L41" s="4" t="inlineStr"/>
       <c r="M41" s="4" t="inlineStr"/>
       <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr">
+      <c r="O41" s="4" t="inlineStr"/>
+      <c r="P41" s="4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="P41" s="4" t="inlineStr"/>
+      <c r="Q41" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P41"/>
+  <autoFilter ref="A1:Q41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3029,7 +3135,7 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4167,10 +4273,16 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
@@ -4245,10 +4357,18 @@
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-28 22:31)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
@@ -2489,52 +2489,125 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>resolucao_conjunta_18_2025</t>
+          <t>normativos_52916</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>571</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>1º de janeiro de 2026.</t>
-        </is>
-      </c>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr"/>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="n">
+        <v>1.888888888888889</v>
+      </c>
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, bem como para a designação e o reconhecimento da</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>dou_pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>resolucao_conjunta_18_2025</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>1º de janeiro de 2026.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>ALTO</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>🔴 APLICÁVEL — Resolução Conjunta nº 18/2025
 **1. Identificação**
@@ -2548,7 +2621,7 @@
 | 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
@@ -2558,160 +2631,165 @@
 | 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
         </is>
       </c>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco C</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
         </is>
       </c>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q32" s="2" t="inlineStr">
         <is>
           <t>dou_html</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>5.307</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
-        </is>
-      </c>
-      <c r="O32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_571_de_28052026</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="4" t="inlineStr"/>
-      <c r="L33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.</t>
+        </is>
+      </c>
       <c r="M33" s="4" t="inlineStr"/>
-      <c r="N33" s="4" t="inlineStr"/>
-      <c r="O33" s="4" t="inlineStr"/>
-      <c r="P33" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, bem como para a designação e o reconhecimento da</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571</t>
+        </is>
+      </c>
+      <c r="P33" s="4" t="inlineStr"/>
       <c r="Q33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
       <c r="Q34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr"/>
@@ -2742,7 +2820,7 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
@@ -2750,9 +2828,9 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -2773,7 +2851,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr"/>
@@ -2781,9 +2859,9 @@
       <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -2804,7 +2882,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
@@ -2835,7 +2913,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -2866,7 +2944,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
@@ -2874,9 +2952,9 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2897,7 +2975,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -2905,9 +2983,9 @@
       <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -2925,8 +3003,70 @@
       </c>
       <c r="Q41" s="4" t="inlineStr"/>
     </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="inlineStr"/>
+      <c r="N43" s="4" t="inlineStr"/>
+      <c r="O43" s="4" t="inlineStr"/>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q41"/>
+  <autoFilter ref="A1:Q43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2999,7 +3139,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3018,11 +3158,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3045,7 +3185,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -3064,7 +3204,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7"/>
@@ -3145,13 +3285,13 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>17</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
@@ -3159,7 +3299,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -3219,7 +3359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3231,7 +3371,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
   </cols>
@@ -4339,41 +4479,43 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>571</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
         <v>3</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="n">
+        <v>1.888888888888889</v>
+      </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -4381,44 +4523,64 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Resolução Conjunta</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I31" s="4" t="inlineStr"/>
       <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>ALTO</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="2" t="inlineStr"/>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
@@ -4427,16 +4589,32 @@
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="4" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>5.307</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+        </is>
+      </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr"/>
@@ -4445,7 +4623,11 @@
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr"/>
       <c r="J33" s="4" t="inlineStr"/>
-      <c r="K33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -4484,8 +4666,44 @@
       <c r="K35" s="4" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr"/>
     </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr"/>
+      <c r="C37" s="4" t="inlineStr"/>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L35"/>
+  <autoFilter ref="A1:L37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4717,7 +4935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -5192,8 +5410,58 @@
       <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-29 19:06)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1946,10 +1946,24 @@
       <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>A norma aborda temas relevantes ao iFood Pago (crédito) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr"/>
+          <t>A norma aborda temas relevantes ao iFood Pago (crédito) mas não menciona explicitamente as entidades do conglomerado. Monitorar.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Altera o leiaute, as instruções de preenchimento e as instruções de programas públicos do documento de código 3040 - Dados de Risco de Crédito, do Sistema de Informações de Créditos (SCR), de que trat</t>
@@ -2019,10 +2033,24 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>A norma aborda temas relevantes ao iFood Pago (banco central) mas não menciona explicitamente as entidades do conglomerado. Monitorar.</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
+          <t>A norma aborda temas relevantes ao iFood Pago (banco central) mas não menciona explicitamente as entidades do conglomerado. Monitorar.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Altera o Regulamento de Avaliação de Desempenho dos Servidores da Carreira de Especialista do Banco Central do Brasil durante o Estágio Probatório.</t>
@@ -2378,8 +2406,7 @@
 |---|---|---|
 | ⚙️ Operacional | 3 | Alterações no Manual Operacional do DICT exigem revisão de fluxos e sistemas. |
 | ⚖️ Regulatório | 3 | Conformidade obrigatória com o Regulamento do Pix e o Manual Operacional do DICT. |
-| 💰 Financeiro | 2 | Potencial impacto financeiro limitado a ajustes operacionais. |
-| 👥 Clientes | 2 | Impacto indireto em clientes, relacionado à continuidade e segurança das operações Pix. |</t>
+| 💰 Financeiro | 2 | Potencial impacto financeiro</t>
         </is>
       </c>
       <c r="M29" s="4" t="inlineStr">
@@ -2461,10 +2488,24 @@
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr"/>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: processo. | Evidências: processo
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: MÉ</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: processo. | Evidências: processo
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: MÉDIO (2/4) | Justificativa: Impacto financeiro moderado: encargo. | Evidências: encargo
+[Impacto em Clientes] Score: ALTO (3/4) | Justificativa: Impacto relevante em clientes (não especificado): usuário, atendimento, lgpd. | Evidências: usuário, atendimento, lgpd
+Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional, Impacto em Clientes. Score médio ponderado: 2.11/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
@@ -2534,10 +2575,23 @@
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr"/>
+          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evi</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros, receita, despesa, orçamento
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.89/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional, Impacto Financeiro. Score médio ponderado: 1.89/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, bem como para a designação e o reconhecimento da</t>
@@ -2582,7 +2636,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>1º de janeiro de 2026.</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2590,50 +2644,54 @@
           <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr"/>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>🔴 APLICÁVEL — Resolução Conjunta nº 18/2025
-**1. Identificação**
-Foi publicada a Resolução Conjunta nº 18, de 28 de novembro de 2025, que dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituiçõ
+          <t>A Res. Conjunta nº 18 não é diretamente aplicável mas deve ser monitorada pois devem implementar e manter política de qualidade das informações prestadas compatível com a sua natureza, o seu porte, a sua complexidade, o seu perfil de risco e o seu modelo de negócio, de forma a a Temas a acompanhar: 
 ### Avaliação de Risco:
-| Pilar | Nível | Motivo |
-|---|---|---|
-| ⚙️ Operacional | 3 | Exige ajustes em processos e sistemas de reporte para atender às novas exigências. |
-| ⚖️ Regulatório | 4 | Norma impõe obrigação direta ao iFood Pago, com risco de sanções em caso de não conformidade. |
-| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e controles, mas sem impacto direto em receitas. |
-| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, processo, controle. | Evidências: procedimento, processo, controle, monitoramento, relatório
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
-| ⚙️ Operacional | 3 | Exige ajustes em processos e sistemas de reporte para atender às novas exigências. |
-| ⚖️ Regulatório | 4 | Norma impõe obrigação direta ao iFood Pago, com risco de sanções em caso de não conformidade. |
-| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e controles, mas sem impacto direto em receitas. |
-| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |</t>
+| ⚙️ Operacional | 3 | Exige mudanças significativas em processos e sistemas de TI para atender às novas dimensões de qualidade. |
+| ⚖️ Regulatório | 4 | Obrigação direta para instituições autorizadas pelo BCB, com impacto em reportes e conformidade. |
+| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e governança, mas sem impacto direto em receitas. |
+| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, processo, controle. | Evidências: procedimento, processo, controle, monitoramento, relatório
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve. | Evidências: deve
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: MÉDIO (2/4) | Justificativa: Impacto moderado em clientes (B2C): usuário. | Evidências: usuário, informação
+Score consolidado: MÉDIO (média ponderada: 2.00/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional. Score médio ponderado: 2.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Dispõe sobre a política de qualidade das informações prestadas na esfera de atuação do Banco Central do Brasil pelas instituições financeiras e demais instituições autorizadas a funcionar pelo Banco C</t>
+          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
@@ -2789,100 +2847,228 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr"/>
+          <t>resolução_conjunta_nº_18_de_28_de_novembro_de_2025</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J35" s="4" t="inlineStr"/>
       <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A Res. Conjunta nº 18 não é diretamente aplicável mas deve ser monitorada pois devem implementar e manter política de qualidade das informações prestadas compatível com a sua natureza, o seu porte, a sua complexidade, o seu perfil de risco e o seu modelo de negócio, de forma a a Temas a acompanhar: </t>
+        </is>
+      </c>
       <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584](https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr"/>
       <c r="Q35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
+          <t>normativos_52917</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="n">
+        <v>1.444444444444444</v>
+      </c>
       <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
-      <c r="O36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api, procedimento. | Evidências: api, procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Fin</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api, procedimento. | Evidências: api, procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.44/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional. Score médio ponderado: 1.44/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
+        </is>
+      </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="inlineStr"/>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
+        </is>
+      </c>
       <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr"/>
-      <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr"/>
       <c r="Q37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
@@ -2890,9 +3076,9 @@
       <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -2913,7 +3099,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr"/>
@@ -2921,9 +3107,9 @@
       <c r="D39" s="4" t="inlineStr"/>
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -2944,7 +3130,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
@@ -2952,9 +3138,9 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
@@ -2975,7 +3161,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -3006,7 +3192,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -3014,9 +3200,9 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -3037,7 +3223,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3045,9 +3231,9 @@
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3065,8 +3251,156 @@
       </c>
       <c r="Q43" s="4" t="inlineStr"/>
     </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52910</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr"/>
+      <c r="N45" s="4" t="inlineStr"/>
+      <c r="O45" s="4" t="inlineStr"/>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr"/>
+      <c r="N47" s="4" t="inlineStr"/>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="inlineStr"/>
+      <c r="Q47" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q43"/>
+  <autoFilter ref="A1:Q47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3135,11 +3469,11 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3158,11 +3492,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3171,7 +3505,7 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -3181,11 +3515,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -3194,7 +3528,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -3204,7 +3538,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7"/>
@@ -3275,7 +3609,7 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -3285,13 +3619,13 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>17</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
@@ -3299,7 +3633,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -3309,13 +3643,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -3359,7 +3693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -4538,26 +4872,28 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G31" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H31" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr"/>
@@ -4631,12 +4967,24 @@
       <c r="L33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="2" t="inlineStr"/>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+        </is>
+      </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
@@ -4645,34 +4993,76 @@
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr"/>
-      <c r="K35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="n">
+        <v>1.444444444444444</v>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="2" t="inlineStr"/>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -4681,7 +5071,11 @@
       <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr"/>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
@@ -4702,8 +5096,62 @@
       <c r="K37" s="4" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr"/>
     </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L37"/>
+  <autoFilter ref="A1:L40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4714,14 +5162,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -4920,8 +5368,46 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H8"/>
+  <autoFilter ref="A2:H9"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -4935,7 +5421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -5460,8 +5946,204 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
     </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>585.7166666666667</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>resolucao_conjunta_18_2025</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 202</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52917</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L10"/>
+  <autoFilter ref="A1:L14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-05-30 00:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$47</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3001,17 +3001,17 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
+          <t>normativos_52919</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>740</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -3019,19 +3019,15 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+      <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -3039,98 +3035,194 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr"/>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K37" s="4" t="inlineStr"/>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
-        </is>
-      </c>
-      <c r="M37" s="4" t="inlineStr"/>
+          <t>A IN BCB nº 740 aplica-se diretamente ao iFood Pago pois revogar a resolução - re nº 1. Menciona explicitamente: open finance. Temas relevantes: pagamento, open finance.
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: revogação. | Evidências: revogação
+[Impacto Financeiro] Score: BAIXO (</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: revogação. | Evidências: revogação
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional, Impacto Regulatório. Score médio ponderado: 2.11/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
-        </is>
-      </c>
-      <c r="P37" s="4" t="inlineStr"/>
-      <c r="Q37" s="4" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>dou_pdf</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_740_de_29052026</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 740 aplica-se diretamente ao iFood Pago pois revogar a resolução - re nº 1. Menciona explicitamente: open finance. Temas relevantes: pagamento, open finance.</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
-      <c r="O38" s="2" t="inlineStr"/>
-      <c r="P38" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
+        </is>
+      </c>
       <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr"/>
-      <c r="P39" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr"/>
       <c r="Q39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
@@ -3161,7 +3253,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -3169,9 +3261,9 @@
       <c r="D41" s="4" t="inlineStr"/>
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -3192,7 +3284,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -3200,9 +3292,9 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -3223,7 +3315,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3254,7 +3346,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
@@ -3285,7 +3377,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -3293,9 +3385,9 @@
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr"/>
       <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
@@ -3316,7 +3408,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
@@ -3324,9 +3416,9 @@
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3334,11 +3426,7 @@
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>Prazo de implementação de 6 meses pode impactar operações</t>
-        </is>
-      </c>
+      <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
       <c r="P46" s="2" t="inlineStr">
@@ -3351,56 +3439,122 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F47" s="4" t="inlineStr"/>
       <c r="G47" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
       <c r="M47" s="4" t="inlineStr"/>
       <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr">
+      <c r="O47" s="4" t="inlineStr"/>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr"/>
+      <c r="N49" s="4" t="inlineStr"/>
+      <c r="O49" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P47" s="4" t="inlineStr"/>
-      <c r="Q47" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr"/>
+      <c r="Q49" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q47"/>
+  <autoFilter ref="A1:Q49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3469,11 +3623,11 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3496,7 +3650,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3528,7 +3682,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -3619,10 +3773,10 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>15</v>
@@ -3633,7 +3787,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -3693,7 +3847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5047,41 +5201,63 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>740</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr"/>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="4" t="inlineStr"/>
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+        </is>
+      </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
@@ -5093,16 +5269,32 @@
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr"/>
       <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
@@ -5111,7 +5303,11 @@
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -5150,8 +5346,44 @@
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
     </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="4" t="inlineStr"/>
+      <c r="C41" s="4" t="inlineStr"/>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L40"/>
+  <autoFilter ref="A1:L42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5421,7 +5653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -6142,8 +6374,58 @@
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
     </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52919</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:L15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-01 17:32)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -573,9 +573,9 @@
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -585,7 +585,7 @@
     <col width="50" customWidth="1" min="14" max="14"/>
     <col width="50" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="23" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3019,7 +3019,11 @@
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
@@ -3032,35 +3036,38 @@
       </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I37" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>2.111111111111111</v>
-      </c>
-      <c r="K37" s="4" t="inlineStr"/>
+        <v>1.25</v>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>A IN BCB nº 740 aplica-se diretamente ao iFood Pago pois revogar a resolução - re nº 1. Menciona explicitamente: open finance. Temas relevantes: pagamento, open finance.
+          <t>A IN BCB nº 740/2026 é aplicável ao iFood Pago como ITP (Iniciador de Transação de Pagamento) e Detentor de Conta no Open Finance. A norma estabelece testes em produção da jornada otimizada. O iFood Pago pode participar opcionalmente como ITP (Art. 2). A oferta obrigatória (Art. 3) aplica-se apenas 
 ### Avaliação de Risco:
-[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
-[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: revogação. | Evidências: revogação
-[Impacto Financeiro] Score: BAIXO (</t>
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Participação opcional; sem mudança de processo obrigatória no momento | Evidências: participação opcional como ITP
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monito</t>
         </is>
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
-[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: revogação. | Evidências: revogação
-[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
-[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
-Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
-Lógica: Pilares ALTOS: Impacto Operacional, Impacto Regulatório. Score médio ponderado: 2.11/4.0 (divisor 4.5)
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Participação opcional; sem mudança de processo obrigatória no momento | Evidências: participação opcional como ITP
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monitorar evolução do papel de Transmissor | Evidências: jornada otimizada, revogação IN 725/2026, Open Finance
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Sem custo de adequação obrigatório no momento | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Sem impacto direto em clientes no momento | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.25/4.0, divisor 4.5)
+Lógica: Score consolidado BAIXO. Pilares: Operacional BAIXO (1), Regulatório MÉDIO (2), Financeiro BAIXO (1), Clientes BAIXO (1). Score médio: 1.25/4.0. Criticidade baixa pois iFood Pago não é Transmissor de Dados, eliminando a obrigação do Art. 3.
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
@@ -3081,7 +3088,7 @@
       </c>
       <c r="Q37" s="4" t="inlineStr">
         <is>
-          <t>dou_pdf</t>
+          <t>corrigido_manualmente</t>
         </is>
       </c>
     </row>
@@ -3101,54 +3108,38 @@
           <t>740</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+      <c r="D38" s="2" t="inlineStr"/>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Verificar texto integral</t>
+          <t>- **22/04/2026**: início de testes em produção (caráter limitado)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I38" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
+          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>A IN BCB nº 740 aplica-se diretamente ao iFood Pago pois revogar a resolução - re nº 1. Menciona explicitamente: open finance. Temas relevantes: pagamento, open finance.</t>
-        </is>
-      </c>
+      <c r="L38" s="2" t="inlineStr"/>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
           <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
         </is>
       </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
-        </is>
-      </c>
+      <c r="O38" s="2" t="inlineStr"/>
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
     </row>
@@ -3623,11 +3614,11 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3682,7 +3673,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -3692,7 +3683,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7"/>
@@ -3763,7 +3754,7 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -3773,10 +3764,10 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D13" s="12" t="n">
         <v>15</v>
@@ -3787,7 +3778,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -3821,7 +3812,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C15" s="12" t="n">
         <v>4</v>
@@ -3853,7 +3844,7 @@
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -5220,10 +5211,10 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>1</v>
@@ -5233,14 +5224,18 @@
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n">
-        <v>2.111111111111111</v>
+        <v>1.25</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr"/>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -5255,12 +5250,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr"/>
@@ -5271,7 +5266,7 @@
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-03 12:02)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -577,9 +577,9 @@
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
     <col width="50" customWidth="1" min="14" max="14"/>
@@ -2530,28 +2530,32 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>resolucao_conjunta_18_2025</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução Conjunta</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr"/>
+          <t>2025-11-28</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
@@ -2564,106 +2568,16 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I31" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>1.888888888888889</v>
+        <v>2</v>
       </c>
       <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.
-### Avaliação de Risco:
-[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
-[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evi</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
-[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
-[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros, receita, despesa, orçamento
-[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
-Score consolidado: BAIXO (média ponderada: 1.89/4.0, divisor 4.5)
-Lógica: Pilares ALTOS: Impacto Operacional, Impacto Financeiro. Score médio ponderado: 1.89/4.0 (divisor 4.5)
-Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, bem como para a designação e o reconhecimento da</t>
-        </is>
-      </c>
-      <c r="O31" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571</t>
-        </is>
-      </c>
-      <c r="P31" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q31" s="4" t="inlineStr">
-        <is>
-          <t>dou_pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>resolucao_conjunta_18_2025</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Resolução Conjunta</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-28</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>A Res. Conjunta nº 18 não é diretamente aplicável mas deve ser monitorada pois devem implementar e manter política de qualidade das informações prestadas compatível com a sua natureza, o seu porte, a sua complexidade, o seu perfil de risco e o seu modelo de negócio, de forma a a Temas a acompanhar: 
 ### Avaliação de Risco:
@@ -2671,7 +2585,7 @@
 [Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
@@ -2689,41 +2603,108 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
+        </is>
+      </c>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>dou_html</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>bc_-_resolução_bcb_n_571_de_28052026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>28/05/2026</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB nº 571 — 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO — monitorar resolução da questão BNDES/FGI</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Imediato (vigência 28/05/2026) — verificar se há impacto após definição do tipo de garantia BNDES/FGI.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>@gabriela.gusella — avaliar o Regulamento FGI para determinar o tipo de garantia e confirmar enquadramento.</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
+          <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, incluindo a constituição de provisão para perdas</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
-        </is>
-      </c>
-      <c r="P32" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q32" s="2" t="inlineStr">
-        <is>
-          <t>dou_html</t>
-        </is>
-      </c>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolução%20BCB&amp;numero=571</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr"/>
+      <c r="Q32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>bc_-_resolução_bcb_n_571_de_28052026</t>
+          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>5.307</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2738,7 +2719,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -2751,27 +2732,27 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I33" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="4" t="inlineStr"/>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>A Res. BCB nº 571 não é diretamente aplicável mas deve ser monitorada pois tornar público o relatório de gestão fiscal do 1º quadrimestre de 2026 desta corte, na forma constante de seu anexo, pertinente ao período de maio de 2025 a abril de 2026. Temas a acompanhar: banco, risco, financeira.</t>
+          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
         </is>
       </c>
       <c r="M33" s="4" t="inlineStr"/>
       <c r="N33" s="4" t="inlineStr">
         <is>
-          <t>Altera a Resolução BCB nº 352, de 23 de novembro de 2023, que dispõe sobre os conceitos e os critérios contábeis aplicáveis a instrumentos financeiros, bem como para a designação e o reconhecimento da</t>
+          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=571</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
         </is>
       </c>
       <c r="P33" s="4" t="inlineStr"/>
@@ -2780,22 +2761,22 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>bc_-_resolução_cmn_n_5307_de_26052026</t>
+          <t>resolução_conjunta_nº_18_de_28_de_novembro_de_2025</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Resolução Conjunta</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2805,7 +2786,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -2827,18 +2808,18 @@
       <c r="K34" s="2" t="inlineStr"/>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>A Res. CMN nº 5.307 não é diretamente aplicável mas deve ser monitorada pois a resolução cmn nº 5. Temas a acompanhar: banco.</t>
+          <t xml:space="preserve">A Res. Conjunta nº 18 não é diretamente aplicável mas deve ser monitorada pois devem implementar e manter política de qualidade das informações prestadas compatível com a sua natureza, o seu porte, a sua complexidade, o seu perfil de risco e o seu modelo de negócio, de forma a a Temas a acompanhar: </t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Altera a Resolução CMN nº 5.300, de 5 de maio de 2026, que estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para aq</t>
+          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
         </is>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5307</t>
+          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584](https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr"/>
@@ -2847,32 +2828,28 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>resolução_conjunta_nº_18_de_28_de_novembro_de_2025</t>
+          <t>normativos_52917</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>572</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2025-11-28</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -2885,79 +2862,16 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I35" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="n">
+        <v>1.444444444444444</v>
+      </c>
       <c r="K35" s="4" t="inlineStr"/>
       <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A Res. Conjunta nº 18 não é diretamente aplicável mas deve ser monitorada pois devem implementar e manter política de qualidade das informações prestadas compatível com a sua natureza, o seu porte, a sua complexidade, o seu perfil de risco e o seu modelo de negócio, de forma a a Temas a acompanhar: </t>
-        </is>
-      </c>
-      <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr">
-        <is>
-          <t>Dispõe sobre a política de qualidade das informações prestadas pelas instituições autorizadas ao Banco Central do Brasil.</t>
-        </is>
-      </c>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584](https://in.gov.br/web/dou/-/resolucao-conjunta-n-18-de-28-de-novembro-de-2025-672006584</t>
-        </is>
-      </c>
-      <c r="P35" s="4" t="inlineStr"/>
-      <c r="Q35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52917</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="n">
-        <v>1.444444444444444</v>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi
 ### Avaliação de Risco:
@@ -2966,7 +2880,7 @@
 [Impacto Fin</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="M35" s="4" t="inlineStr">
         <is>
           <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api, procedimento. | Evidências: api, procedimento
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -2977,82 +2891,82 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr">
+      <c r="O35" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
         </is>
       </c>
-      <c r="P36" s="2" t="inlineStr">
+      <c r="P35" s="4" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="Q36" s="2" t="inlineStr">
+      <c r="Q35" s="4" t="inlineStr">
         <is>
           <t>ementa</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>normativos_52919</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>740</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="J37" s="4" t="n">
+      <c r="J36" s="2" t="n">
         <v>1.25</v>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>A IN BCB nº 740/2026 é aplicável ao iFood Pago como ITP (Iniciador de Transação de Pagamento) e Detentor de Conta no Open Finance. A norma estabelece testes em produção da jornada otimizada. O iFood Pago pode participar opcionalmente como ITP (Art. 2). A oferta obrigatória (Art. 3) aplica-se apenas 
 ### Avaliação de Risco:
@@ -3060,7 +2974,7 @@
 [Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monito</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Participação opcional; sem mudança de processo obrigatória no momento | Evidências: participação opcional como ITP
 [Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monitorar evolução do papel de Transmissor | Evidências: jornada otimizada, revogação IN 725/2026, Open Finance
@@ -3071,60 +2985,119 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>corrigido_manualmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>bc_-_instrução_normativa_bcb_n_740_de_29052026</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>- **22/04/2026**: início de testes em produção (caráter limitado)</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
       <c r="N37" s="4" t="inlineStr">
         <is>
           <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
         </is>
       </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
-        </is>
-      </c>
-      <c r="P37" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="Q37" s="4" t="inlineStr">
-        <is>
-          <t>corrigido_manualmente</t>
-        </is>
-      </c>
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr"/>
+      <c r="Q37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>bc_-_instrução_normativa_bcb_n_740_de_29052026</t>
+          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>- **22/04/2026**: início de testes em produção (caráter limitado)</t>
+          <t>Verificar texto integral</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
       <c r="I38" s="7" t="inlineStr">
         <is>
           <t>BAIXO</t>
@@ -3132,88 +3105,60 @@
       </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr"/>
+          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
+        </is>
+      </c>
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+          <t>normativos_52913</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr"/>
+      <c r="C39" s="4" t="inlineStr"/>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr"/>
       <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="inlineStr">
-        <is>
-          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
-        </is>
-      </c>
+      <c r="L39" s="4" t="inlineStr"/>
       <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
-        </is>
-      </c>
-      <c r="P39" s="4" t="inlineStr"/>
+      <c r="N39" s="4" t="inlineStr"/>
+      <c r="O39" s="4" t="inlineStr"/>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
@@ -3244,7 +3189,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -3275,7 +3220,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -3283,9 +3228,9 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -3306,7 +3251,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3337,7 +3282,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
@@ -3368,7 +3313,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -3399,7 +3344,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
@@ -3407,9 +3352,9 @@
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3430,7 +3375,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52915</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
@@ -3448,7 +3393,11 @@
       <c r="J47" s="4" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+        </is>
+      </c>
       <c r="N47" s="4" t="inlineStr"/>
       <c r="O47" s="4" t="inlineStr"/>
       <c r="P47" s="4" t="inlineStr">
@@ -3461,27 +3410,41 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52916</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros, receita, despesa, orçamento
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.89/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional, Impacto Financeiro. Score médio ponderado: 1.89/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr"/>
@@ -3556,7 +3519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3683,7 +3646,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7"/>
@@ -3736,17 +3699,17 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Apr/2026</t>
+          <t>28/05/2</t>
         </is>
       </c>
       <c r="B12" s="13" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="13" t="n">
         <v>1</v>
-      </c>
-      <c r="D12" s="13" t="n">
-        <v>0</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -3760,17 +3723,17 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>May/2026</t>
+          <t>Apr/2026</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
@@ -3778,23 +3741,23 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Nov/2025</t>
+          <t>May/2026</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -3808,17 +3771,33 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
+          <t>Nov/2025</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" s="12" t="n">
+      <c r="B16" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C16" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="12" t="n">
-        <v>0</v>
+      <c r="D16" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3851,8 +3830,8 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4958,17 +4937,17 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução Conjunta</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -4980,21 +4959,21 @@
         <v>3</v>
       </c>
       <c r="F30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="H30" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>1.888888888888889</v>
+        <v>2</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -5002,17 +4981,17 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>571</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+          <t>Resolução BCB nº 571 — 28/05/2026</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -5020,43 +4999,37 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr"/>
+          <t>BAIXO — monitorar resolução da questão BNDES/FGI</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Imediato (vigência 28/05/2026) — verificar se há impacto após definição do tipo de garantia BNDES/FGI.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>5.307</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -5072,7 +5045,7 @@
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr"/>
@@ -5080,17 +5053,17 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Resolução Conjunta</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -5114,17 +5087,17 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>572</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 2025</t>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -5132,15 +5105,25 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="n">
+        <v>1.444444444444444</v>
+      </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
@@ -5148,29 +5131,29 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>740</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>1</v>
@@ -5180,14 +5163,18 @@
       </c>
       <c r="I35" s="4" t="inlineStr"/>
       <c r="J35" s="4" t="n">
-        <v>1.444444444444444</v>
+        <v>1.25</v>
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr"/>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -5202,60 +5189,46 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="n">
-        <v>1.25</v>
-      </c>
+      <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
+      <c r="L36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>740</t>
+          <t>572</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr"/>
@@ -5272,24 +5245,12 @@
       <c r="L37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
@@ -5298,11 +5259,7 @@
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="K38" s="2" t="inlineStr"/>
       <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
@@ -5362,10 +5319,14 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr"/>
       <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
@@ -5374,7 +5335,11 @@
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L42" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -5648,7 +5613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -5657,11 +5622,11 @@
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="31" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -6419,8 +6384,554 @@
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
     </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>test_validacao_001</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Teste de validação pós-correção</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>315.35</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>feedback_test_validacao</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>test_validacao_001</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Teste de validação pós-correção</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>316.65</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>feedback_test_validacao</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>test_validacao_001</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Teste de validação pós-correção</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>317.4333333333333</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>feedback_test_validacao</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>test_feedback_recebido_001</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB nº 569</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>197.4333333333333</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>slack_msg_001</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>test_validacao_001</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Teste de validação pós-correção</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>319.1</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>feedback_test_validacao</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>resolucao_cmn_5304</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>5304</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN nº 5304</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>feedback_1</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>resolucao_cmn_5304</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>5304</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN nº 5304</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>feedback_1</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 738, de 27/05/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>feedback_confirmacao_738</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52919</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 740, de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="n">
+        <v>75</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1780317708.145359</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52919</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 740, de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1780317708.145359</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L15"/>
+  <autoFilter ref="A1:L25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-04 00:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q49"/>
+  <dimension ref="A1:Q51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3127,69 +3127,160 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr"/>
+          <t>normativos_52920</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
       <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr"/>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr"/>
-      <c r="J39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="inlineStr"/>
-      <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A IN BCB nº 741 não é diretamente aplicável mas deve ser monitorada pois altera as instruções normativas bcb ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do padrão contábil das instituições reguladas pelo banco cen Temas a acompanhar: banco,
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação, dever, deve. | Evidências: liquidação, dever, </t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação, dever, deve. | Evidências: liquidação, dever, deve
+[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto mínimo em clientes (não especificado). | Evidências: comunicado
+Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Regulatório, Impacto Financeiro. Score médio ponderado: 2.11/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>Altera as Instruções Normativas BCB ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Reguladas pelo Banco Cen</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=741</t>
+        </is>
+      </c>
       <c r="P39" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q39" s="4" t="inlineStr"/>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>dou_pdf</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_741_de_03062026</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 741 não é diretamente aplicável mas deve ser monitorada pois altera as instruções normativas bcb ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do padrão contábil das instituições reguladas pelo banco cen Temas a acompanhar: banco,</t>
+        </is>
+      </c>
       <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Altera as Instruções Normativas BCB ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Reguladas pelo Banco Cen</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=741](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=741</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr"/>
       <c r="Q40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr"/>
@@ -3220,7 +3311,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -3228,9 +3319,9 @@
       <c r="D42" s="2" t="inlineStr"/>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -3251,7 +3342,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3259,9 +3350,9 @@
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3282,7 +3373,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
@@ -3313,7 +3404,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -3344,7 +3435,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
@@ -3352,9 +3443,9 @@
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3375,7 +3466,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
@@ -3383,9 +3474,9 @@
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
@@ -3393,11 +3484,7 @@
       <c r="J47" s="4" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr"/>
       <c r="L47" s="4" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr">
-        <is>
-          <t>Prazo de implementação de 6 meses pode impactar operações</t>
-        </is>
-      </c>
+      <c r="M47" s="4" t="inlineStr"/>
       <c r="N47" s="4" t="inlineStr"/>
       <c r="O47" s="4" t="inlineStr"/>
       <c r="P47" s="4" t="inlineStr">
@@ -3410,33 +3497,99 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr"/>
-      <c r="M48" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr"/>
+      <c r="O49" s="4" t="inlineStr"/>
+      <c r="P49" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -3447,68 +3600,68 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
-      <c r="N48" s="2" t="inlineStr"/>
-      <c r="O48" s="2" t="inlineStr"/>
-      <c r="P48" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="Q48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="Q50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>normativos_52918</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>739</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
+      <c r="G51" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H49" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr"/>
+      <c r="N51" s="4" t="inlineStr"/>
+      <c r="O51" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P49" s="4" t="inlineStr"/>
-      <c r="Q49" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr"/>
+      <c r="Q51" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q49"/>
+  <autoFilter ref="A1:Q51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3519,7 +3672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3581,7 +3734,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>46%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3600,11 +3753,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3627,7 +3780,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -3636,7 +3789,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -3741,23 +3894,23 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>May/2026</t>
+          <t>Jun/2026</t>
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -3771,32 +3924,48 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>Nov/2025</t>
+          <t>May/2026</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D15" s="12" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
+          <t>Nov/2025</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B17" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C17" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D17" s="12" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3817,7 +3986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5245,30 +5414,68 @@
       <c r="L37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="n">
+        <v>2.111111111111111</v>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="4" t="inlineStr"/>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr"/>
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr"/>
@@ -5277,7 +5484,11 @@
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr"/>
       <c r="J39" s="4" t="inlineStr"/>
-      <c r="K39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
@@ -5319,14 +5530,10 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr"/>
       <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C42" s="2" t="inlineStr"/>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
@@ -5335,15 +5542,55 @@
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr"/>
+      <c r="C43" s="4" t="inlineStr"/>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L42"/>
+  <autoFilter ref="A1:L44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5613,7 +5860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -6930,8 +7177,58 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52920</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L25"/>
+  <autoFilter ref="A1:L26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-09 19:59)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3280,69 +3280,168 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr"/>
+          <t>normativos_52921</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
       <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr"/>
-      <c r="J41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>1.222222222222222</v>
+      </c>
       <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="4" t="inlineStr"/>
-      <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 742 não é diretamente aplicável mas deve ser monitorada pois divulga a versão 8.3 do manual operacional do diretório de identificadores de contas transacionais (dict), que compõe o regulamento do pix. Temas a acompanhar: pix.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Alterações no DICT podem exigir ajustes técnicos e operacionais no Pix e produtos correlatos. |
+| ⚖️ Regulatório | 3 | O DICT é parte do Regulamento do Pix, e mudanças podem impactar a conformidade regulatória. |
+| 💰 Financeiro | 2 | Potencial impacto em custos operacionais para implementação de ajustes. |
+| 👥 Clientes | 2 | Possíveis alterações na experiência do cliente em relação ao uso do Pix. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: MÉDIO (2/4) | Justificativa: Impacto moderado em clientes (não especificado): sac. | Evidências: sac
+Score consolidado: BAIXO (média ponderada: 1.22/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.22/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>Divulga a versão 8.3 do Manual Operacional do Diretório de Identificadores de Contas Transacionais (DICT), que compõe o Regulamento do Pix.</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=742</t>
+        </is>
+      </c>
       <c r="P41" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q41" s="4" t="inlineStr"/>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="Q41" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_742_de_09062026</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 742 não é diretamente aplicável mas deve ser monitorada pois divulga a versão 8.3 do manual operacional do diretório de identificadores de contas transacionais (dict), que compõe o regulamento do pix. Temas a acompanhar: pix.</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
-      <c r="O42" s="2" t="inlineStr"/>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Divulga a versão 8.3 do Manual Operacional do Diretório de Identificadores de Contas Transacionais (DICT), que compõe o Regulamento do Pix.</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=742](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=742</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
       <c r="Q42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr"/>
@@ -3373,7 +3472,7 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
@@ -3381,9 +3480,9 @@
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -3404,7 +3503,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -3412,9 +3511,9 @@
       <c r="D45" s="4" t="inlineStr"/>
       <c r="E45" s="4" t="inlineStr"/>
       <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
@@ -3435,7 +3534,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
@@ -3466,7 +3565,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
@@ -3497,7 +3596,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
@@ -3505,9 +3604,9 @@
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -3528,7 +3627,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3536,9 +3635,9 @@
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
@@ -3546,11 +3645,7 @@
       <c r="J49" s="4" t="inlineStr"/>
       <c r="K49" s="4" t="inlineStr"/>
       <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr">
-        <is>
-          <t>Prazo de implementação de 6 meses pode impactar operações</t>
-        </is>
-      </c>
+      <c r="M49" s="4" t="inlineStr"/>
       <c r="N49" s="4" t="inlineStr"/>
       <c r="O49" s="4" t="inlineStr"/>
       <c r="P49" s="4" t="inlineStr">
@@ -3563,33 +3658,99 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
       <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr"/>
-      <c r="M50" s="2" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>Prazo de implementação de 6 meses pode impactar operações</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr"/>
+      <c r="O51" s="4" t="inlineStr"/>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -3600,68 +3761,68 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
-      <c r="P50" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr"/>
+      <c r="P52" s="2" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="Q50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="Q52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>normativos_52918</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>739</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>2026-05-29</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
-      <c r="G51" s="9" t="inlineStr">
+      <c r="G53" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>ALTA</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr"/>
-      <c r="J51" s="4" t="inlineStr"/>
-      <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr">
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr"/>
+      <c r="M53" s="4" t="inlineStr"/>
+      <c r="N53" s="4" t="inlineStr"/>
+      <c r="O53" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P51" s="4" t="inlineStr"/>
-      <c r="Q51" s="4" t="inlineStr"/>
+      <c r="P53" s="4" t="inlineStr"/>
+      <c r="Q53" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q51"/>
+  <autoFilter ref="A1:Q53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3734,7 +3895,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3753,11 +3914,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3780,7 +3941,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -3799,7 +3960,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7"/>
@@ -3894,7 +4055,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
@@ -3904,13 +4065,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -3986,7 +4147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5492,30 +5653,68 @@
       <c r="L39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="n">
+        <v>1.222222222222222</v>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr"/>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr"/>
@@ -5524,7 +5723,11 @@
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr"/>
       <c r="J41" s="4" t="inlineStr"/>
-      <c r="K41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L41" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
@@ -5566,14 +5769,10 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr"/>
       <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C44" s="2" t="inlineStr"/>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -5582,15 +5781,55 @@
       <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr"/>
+      <c r="C45" s="4" t="inlineStr"/>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L44"/>
+  <autoFilter ref="A1:L46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5860,7 +6099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -7227,8 +7466,58 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
     </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52921</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L26"/>
+  <autoFilter ref="A1:L27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-10 14:00)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6099,10 +6099,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
@@ -7516,8 +7516,446 @@
       <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="4" t="inlineStr"/>
     </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52920</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>C07SA5U2VPF_1781016185.927369</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Abreu</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52921</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>C07SA5U2VPF_1781035173.652689</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Abreu</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>bc___instru__o_normativa_bcb_n__742_de_09_06_2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>27.23333333333333</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1781040255.150709</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>U097D4HTGJY</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>in_bcb_n__742</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>IN BCB nº 742</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>26.63333333333333</v>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1781040292.442009</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>U097D4HTGJY</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__740</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 740</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>12069.73333333333</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1780317708.145359</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Abreu</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__741_de_03_06_2026</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr"/>
+      <c r="C33" s="4" t="inlineStr"/>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>18.41666666666667</v>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>C07SA5U2VPF_1781016185.927369</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Abreu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__742_de_09_06_2026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 742 de 09/06/2026</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>18.45</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>feedback_recebido</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>C07SA5U2VPF_1781035173.652689</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Abreu</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52921</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>IN BCB nº 742/2026 — Manual DICT v8.3</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1781040255.150709</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52921</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>IN BCB nº 742/2026 — Manual DICT v8.3</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F36" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>C09F6UUL9TK_1781040292.442009</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Giovanna Batistutti</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L27"/>
+  <autoFilter ref="A1:L36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-10 20:00)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -149,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,7 +200,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2587,14 +2586,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>| Pilar | Nível | Motivo |
-|---|---|---|
-| ⚙️ Operacional | 3 | Exige mudanças significativas em processos e sistemas de TI para atender às novas dimensões de qualidade. |
-| ⚖️ Regulatório | 4 | Obrigação direta para instituições autorizadas pelo BCB, com impacto em reportes e conformidade. |
-| 💰 Financeiro | 2 | Custos moderados para implementação de sistemas e governança, mas sem impacto direto em receitas. |
-| 👥 Clientes | 1 | Impacto indireto, sem alteração na experiência do cliente. |
---- Cálculo determinístico ---
-[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, processo, controle. | Evidências: procedimento, processo, controle, monitoramento, relatório
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, processo, controle. | Evidências: procedimento, processo, controle, monitoramento, relatório
 [Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve. | Evidências: deve
 [Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
 [Impacto em Clientes] Score: MÉDIO (2/4) | Justificativa: Impacto moderado em clientes (B2C): usuário. | Evidências: usuário, informação
@@ -2976,12 +2968,19 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Participação opcional; sem mudança de processo obrigatória no momento | Evidências: participação opcional como ITP
-[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monitorar evolução do papel de Transmissor | Evidências: jornada otimizada, revogação IN 725/2026, Open Finance
-[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Sem custo de adequação obrigatório no momento | Evidências: nenhuma evidência direta
-[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Sem impacto direto em clientes no momento | Evidências: nenhuma evidência direta
-Score consolidado: BAIXO (média ponderada: 1.25/4.0, divisor 4.5)
-Lógica: Score consolidado BAIXO. Pilares: Operacional BAIXO (1), Regulatório MÉDIO (2), Financeiro BAIXO (1), Clientes BAIXO (1). Score médio: 1.25/4.0. Criticidade baixa pois iFood Pago não é Transmissor de Dados, eliminando a obrigação do Art. 3.
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Necessidade de adequação técnica para testes em produção e integração com APIs do Open Finance. |
+| ⚖️ Regulatório | 4 | Obrigação normativa vinculada ao Open Finance, com impacto direto na conformidade regulatória. |
+| 💰 Financeiro | 2 | Custos moderados para implementação e testes, mas sem impacto significativo no modelo de negócios. |
+| 👥 Clientes | 3 | Potencial impacto na experiência do cliente durante os testes, exigindo comunicação clara e gestão de consentimento. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
@@ -3336,10 +3335,10 @@
         <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
-| ⚙️ Operacional | 3 | Alterações no DICT podem exigir ajustes técnicos e operacionais no Pix e produtos correlatos. |
-| ⚖️ Regulatório | 3 | O DICT é parte do Regulamento do Pix, e mudanças podem impactar a conformidade regulatória. |
-| 💰 Financeiro | 2 | Potencial impacto em custos operacionais para implementação de ajustes. |
-| 👥 Clientes | 2 | Possíveis alterações na experiência do cliente em relação ao uso do Pix. |
+| ⚙️ Operacional | 3 | Alterações no DICT podem exigir ajustes em sistemas e processos operacionais. |
+| ⚖️ Regulatório | 4 | Conformidade com o DICT é obrigatória para participantes do Pix. |
+| 💰 Financeiro | 2 | Risco financeiro moderado em caso de não conformidade, como multas ou sanções. |
+| 👥 Clientes | 3 | Impacto na experiência do cliente em caso de falhas no registro ou portabilidade de chaves. |
 --- Cálculo determinístico ---
 [Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -3707,11 +3706,7 @@
       <c r="J51" s="4" t="inlineStr"/>
       <c r="K51" s="4" t="inlineStr"/>
       <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr">
-        <is>
-          <t>Prazo de implementação de 6 meses pode impactar operações</t>
-        </is>
-      </c>
+      <c r="M51" s="4" t="inlineStr"/>
       <c r="N51" s="4" t="inlineStr"/>
       <c r="O51" s="4" t="inlineStr"/>
       <c r="P51" s="4" t="inlineStr">
@@ -3750,17 +3745,7 @@
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento, relatório, fluxo. | Evidências: procedimento, relatório, fluxo
-[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
-[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros, receita, despesa, orçamento
-[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
-Score consolidado: BAIXO (média ponderada: 1.89/4.0, divisor 4.5)
-Lógica: Pilares ALTOS: Impacto Operacional, Impacto Financeiro. Score médio ponderado: 1.89/4.0 (divisor 4.5)
-Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
-        </is>
-      </c>
+      <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr"/>
       <c r="O52" s="2" t="inlineStr"/>
       <c r="P52" s="2" t="inlineStr">
@@ -6099,21 +6084,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="31" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -6181,33 +6166,35 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>normativos_52913_test</t>
+          <t>normativos_52920</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>5306</t>
+          <t>741</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5306 - Teste de auditoria</t>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>inicial</t>
@@ -6215,12 +6202,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>CRÍTICO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
@@ -6229,63 +6216,57 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913_test</t>
+          <t>normativos_52919</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>5306</t>
+          <t>740</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Resolução CMN nº 5306 - Teste de auditoria</t>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="n">
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="4" t="inlineStr"/>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>reanalise_feedback</t>
+          <t>inicial</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>feedback_1</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52918</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -6295,12 +6276,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>738</t>
+          <t>739</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -6312,7 +6293,7 @@
         <v>50</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>326.95</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -6322,7 +6303,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -6331,44 +6312,48 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52917</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>738</t>
+          <t>572</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 738 de 27/05/2026</t>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>NÃO APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="F5" s="17" t="n">
         <v>50</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>329.05</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>inicial</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr"/>
@@ -6377,44 +6362,48 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>normativos_52914</t>
+          <t>normativos_52921</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Resolução CMN</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>5.307</t>
+          <t>742</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução CMN N° 5.307 de 26/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>NÃO APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="F6" s="17" t="n">
         <v>50</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>329.0833333333333</v>
+        <v>0</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>inicial</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -6423,7 +6412,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52920</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -6433,12 +6422,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>738</t>
+          <t>741</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB N° 738 de 27/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -6446,42 +6435,34 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="F7" s="18" t="n">
-        <v>85</v>
+      <c r="F7" s="17" t="n">
+        <v>50</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>reanalise_feedback</t>
+          <t>inicial</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>feedback_e2e_test_001</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>instrucao_normativa_bcb_722</t>
+          <t>normativos_52919</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -6491,12 +6472,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>740</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instrução Normativa BCB nº 722, de 13 de abril de </t>
+          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -6505,9 +6486,11 @@
         </is>
       </c>
       <c r="F8" s="17" t="n">
-        <v>60</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>inicial</t>
@@ -6515,12 +6498,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>ALTO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -6529,46 +6512,44 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>resolucao_conjunta_18_2025</t>
+          <t>normativos_52918</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>739</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 202</t>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="F9" s="17" t="n">
-        <v>60</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
           <t>inicial</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>ALTO</t>
-        </is>
-      </c>
+      <c r="I9" s="4" t="inlineStr"/>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr"/>
@@ -6577,7 +6558,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52917</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -6587,12 +6568,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>571</t>
+          <t>572</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -6601,7 +6582,7 @@
         </is>
       </c>
       <c r="F10" s="17" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
@@ -6618,1344 +6599,14 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52916</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>571</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>585.7166666666667</v>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
-      <c r="L11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>resolucao_conjunta_18_2025</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Resolução Conjunta</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Resolução Conjunta nº 18, de 28 de novembro de 202</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F12" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52917</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F14" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52919</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F15" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>test_validacao_001</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Teste de validação pós-correção</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>315.35</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>feedback_test_validacao</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>test_validacao_001</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Teste de validação pós-correção</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F17" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>316.65</v>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>feedback_test_validacao</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>test_validacao_001</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Teste de validação pós-correção</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>317.4333333333333</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>feedback_test_validacao</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>test_feedback_recebido_001</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Resolução BCB nº 569</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>197.4333333333333</v>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>slack_msg_001</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>test_validacao_001</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Teste de validação pós-correção</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F20" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G20" s="2" t="n">
-        <v>319.1</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>feedback_test_validacao</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5304</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>5304</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Resolução CMN nº 5304</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F21" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>feedback_1</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>resolucao_cmn_5304</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>5304</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Resolução CMN nº 5304</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F22" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>feedback_1</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52915</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>738</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 738, de 27/05/2026</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F23" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-27</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>feedback_confirmacao_738</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52919</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 740, de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F24" s="18" t="n">
-        <v>75</v>
-      </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1780317708.145359</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52919</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 740, de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F25" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1780317708.145359</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52920</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F26" s="17" t="n">
-        <v>65</v>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52921</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>742</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F27" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr"/>
-      <c r="L27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52920</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 741 de 03/06/2026</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F28" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>C07SA5U2VPF_1781016185.927369</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Abreu</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52921</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>742</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 742 de 09/06/2026</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F29" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>C07SA5U2VPF_1781035173.652689</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Abreu</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>bc___instru__o_normativa_bcb_n__742_de_09_06_2026</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F30" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>27.23333333333333</v>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1781040255.150709</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>U097D4HTGJY</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>in_bcb_n__742</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>IN BCB nº 742</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F31" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>26.63333333333333</v>
-      </c>
-      <c r="H31" s="4" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I31" s="4" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1781040292.442009</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>U097D4HTGJY</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>instru__o_normativa_bcb_n__740</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 740</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F32" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>12069.73333333333</v>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1780317708.145359</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Abreu</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>instru__o_normativa_bcb_n__741_de_03_06_2026</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr"/>
-      <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 741 de 03/06/2026</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F33" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>18.41666666666667</v>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr"/>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t>C07SA5U2VPF_1781016185.927369</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Abreu</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>instru__o_normativa_bcb_n__742_de_09_06_2026</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 742 de 09/06/2026</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="F34" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>18.45</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>feedback_recebido</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>C07SA5U2VPF_1781035173.652689</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Abreu</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52921</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>742</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>IN BCB nº 742/2026 — Manual DICT v8.3</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F35" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr"/>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1781040255.150709</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52921</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>742</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>IN BCB nº 742/2026 — Manual DICT v8.3</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F36" s="18" t="n">
-        <v>85</v>
-      </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>reanalise_feedback</t>
-        </is>
-      </c>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>C09F6UUL9TK_1781040292.442009</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Giovanna Batistutti</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L36"/>
+  <autoFilter ref="A1:L10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-11 11:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3440,69 +3440,161 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
+          <t>normativos_52922</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
       <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>1.333333333333333</v>
+      </c>
       <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="4" t="inlineStr"/>
-      <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: requerimento. | Evidências: requerimento
+[Impacto Financei</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: requerimento. | Evidências: requerimento
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.33/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.33/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
+        </is>
+      </c>
       <c r="P43" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q43" s="4" t="inlineStr"/>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_573_de_10062026</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc</t>
+        </is>
+      </c>
       <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr"/>
-      <c r="O44" s="2" t="inlineStr"/>
-      <c r="P44" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr"/>
       <c r="Q44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr"/>
@@ -3533,7 +3625,7 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr"/>
@@ -3541,9 +3633,9 @@
       <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -3564,7 +3656,7 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
@@ -3572,9 +3664,9 @@
       <c r="D47" s="4" t="inlineStr"/>
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
@@ -3595,7 +3687,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
@@ -3626,7 +3718,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3657,7 +3749,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
@@ -3665,9 +3757,9 @@
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -3688,7 +3780,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr"/>
@@ -3696,9 +3788,9 @@
       <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
@@ -3719,29 +3811,21 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr"/>
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
@@ -3758,56 +3842,126 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr"/>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr"/>
       <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F53" s="4" t="inlineStr"/>
       <c r="G53" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H53" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="4" t="inlineStr"/>
       <c r="J53" s="4" t="inlineStr"/>
       <c r="K53" s="4" t="inlineStr"/>
       <c r="L53" s="4" t="inlineStr"/>
       <c r="M53" s="4" t="inlineStr"/>
       <c r="N53" s="4" t="inlineStr"/>
-      <c r="O53" s="4" t="inlineStr">
+      <c r="O53" s="4" t="inlineStr"/>
+      <c r="P53" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr"/>
+      <c r="N55" s="4" t="inlineStr"/>
+      <c r="O55" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P53" s="4" t="inlineStr"/>
-      <c r="Q53" s="4" t="inlineStr"/>
+      <c r="P55" s="4" t="inlineStr"/>
+      <c r="Q55" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q53"/>
+  <autoFilter ref="A1:Q55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3880,7 +4034,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -3899,11 +4053,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -3945,7 +4099,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7"/>
@@ -4040,7 +4194,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14">
@@ -4050,13 +4204,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -4132,7 +4286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5716,30 +5870,68 @@
       <c r="L41" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="n">
+        <v>1.333333333333333</v>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="4" t="inlineStr"/>
-      <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr"/>
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr"/>
@@ -5748,7 +5940,11 @@
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr"/>
       <c r="J43" s="4" t="inlineStr"/>
-      <c r="K43" s="4" t="inlineStr"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L43" s="4" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
@@ -5790,14 +5986,10 @@
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr"/>
       <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C46" s="2" t="inlineStr"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
@@ -5806,15 +5998,55 @@
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="2" t="inlineStr"/>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L46"/>
+  <autoFilter ref="A1:L48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6084,7 +6316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6605,8 +6837,58 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
     </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52922</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L10"/>
+  <autoFilter ref="A1:L11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-11 19:05)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2968,12 +2968,216 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Participação opcional; sem mudança de processo obrigatória no momento | Evidências: participação opcional como ITP
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Nova obrigação para Transmissores de Dados (iFood Pago não é); monitorar evolução do papel de Transmissor | Evidências: jornada otimizada, revogação IN 725/2026, Open Finance
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Sem custo de adequação obrigatório no momento | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Sem impacto direto em clientes no momento | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.25/4.0, divisor 4.5)
+Lógica: Score consolidado BAIXO. Pilares: Operacional BAIXO (1), Regulatório MÉDIO (2), Financeiro BAIXO (1), Clientes BAIXO (1). Score médio: 1.25/4.0. Criticidade baixa pois iFood Pago não é Transmissor de Dados, eliminando a obrigação do Art. 3.
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="Q36" s="2" t="inlineStr">
+        <is>
+          <t>corrigido_manualmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>bc_-_instrução_normativa_bcb_n_740_de_29052026</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>- **22/04/2026**: início de testes em produção (caráter limitado)</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="4" t="inlineStr"/>
+      <c r="M37" s="4" t="inlineStr"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr"/>
+      <c r="P37" s="4" t="inlineStr"/>
+      <c r="Q37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr"/>
+      <c r="Q38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52920</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>741</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A IN BCB nº 741 não é diretamente aplicável mas deve ser monitorada pois altera as instruções normativas bcb ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do padrão contábil das instituições reguladas pelo banco cen Temas a acompanhar: banco,
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação, dever, deve. | Evidências: liquidação, dever, </t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
-| ⚙️ Operacional | 3 | Necessidade de adequação técnica para testes em produção e integração com APIs do Open Finance. |
-| ⚖️ Regulatório | 4 | Obrigação normativa vinculada ao Open Finance, com impacto direto na conformidade regulatória. |
-| 💰 Financeiro | 2 | Custos moderados para implementação e testes, mas sem impacto significativo no modelo de negócios. |
-| 👥 Clientes | 3 | Potencial impacto na experiência do cliente durante os testes, exigindo comunicação clara e gestão de consentimento. |
+| ⚙️ Operacional | 3 | Alterações podem demandar ajustes em sistemas contábeis e processos internos. |
+| ⚖️ Regulatório | 4 | Impacto direto em reportes regulatórios e conformidade com normas do BCB. |
+| 💰 Financeiro | 2 | Possibilidade de custos associados a ajustes e reclassificações. |
+| 👥 Clientes | 1 | Impacto indireto, sem efeito direto na experiência do cliente. |
 --- Cálculo determinístico ---
 [Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -2984,210 +3188,6 @@
 Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
         </is>
       </c>
-      <c r="N36" s="2" t="inlineStr">
-        <is>
-          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=740</t>
-        </is>
-      </c>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="inlineStr">
-        <is>
-          <t>corrigido_manualmente</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>bc_-_instrução_normativa_bcb_n_740_de_29052026</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>- **22/04/2026**: início de testes em produção (caráter limitado)</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB nº 740 — 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL (participação opcional como ITP; sem obrigação como Transmissor de Dados)</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr"/>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="4" t="inlineStr"/>
-      <c r="M37" s="4" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr">
-        <is>
-          <t>Estabelece as orientações, as condições e os prazos para a realização de testes em produção pelas instituições participantes relativos ao compartilhamento de serviço otimizado de iniciação de transaçã</t>
-        </is>
-      </c>
-      <c r="O37" s="4" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr"/>
-      <c r="Q37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>bc_-_resolução_bcb_n_572_de_29052026</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr"/>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>A Res. BCB nº 572 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – matpf, para incluir os instrumentos  Temas a acompanhar: capi</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Altera a Resolução BCB nº 102, de 7 de junho de 2021, para atualizar os procedimentos relativos à apuração do montante a ser alocado em títulos públicos federais – MATPF, para incluir os instrumentos </t>
-        </is>
-      </c>
-      <c r="O38" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=572</t>
-        </is>
-      </c>
-      <c r="P38" s="2" t="inlineStr"/>
-      <c r="Q38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52920</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr"/>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I39" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="n">
-        <v>2.111111111111111</v>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A IN BCB nº 741 não é diretamente aplicável mas deve ser monitorada pois altera as instruções normativas bcb ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do padrão contábil das instituições reguladas pelo banco cen Temas a acompanhar: banco,
-### Avaliação de Risco:
-[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
-[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação, dever, deve. | Evidências: liquidação, dever, </t>
-        </is>
-      </c>
-      <c r="M39" s="4" t="inlineStr">
-        <is>
-          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
-[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação, dever, deve. | Evidências: liquidação, dever, deve
-[Impacto Financeiro] Score: ALTO (3/4) | Justificativa: Impacto financeiro relevante: taxa, juros. | Evidências: taxa, juros
-[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto mínimo em clientes (não especificado). | Evidências: comunicado
-Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
-Lógica: Pilares ALTOS: Impacto Regulatório, Impacto Financeiro. Score médio ponderado: 2.11/4.0 (divisor 4.5)
-Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
-        </is>
-      </c>
       <c r="N39" s="4" t="inlineStr">
         <is>
           <t>Altera as Instruções Normativas BCB ns. 428, 429 e 433, todas de 1º de dezembro de 2023, que definem rubricas contábeis do elenco de contas do Padrão Contábil das Instituições Reguladas pelo Banco Cen</t>
@@ -3335,10 +3335,10 @@
         <is>
           <t>| Pilar | Nível | Motivo |
 |---|---|---|
-| ⚙️ Operacional | 3 | Alterações no DICT podem exigir ajustes em sistemas e processos operacionais. |
-| ⚖️ Regulatório | 4 | Conformidade com o DICT é obrigatória para participantes do Pix. |
-| 💰 Financeiro | 2 | Risco financeiro moderado em caso de não conformidade, como multas ou sanções. |
-| 👥 Clientes | 3 | Impacto na experiência do cliente em caso de falhas no registro ou portabilidade de chaves. |
+| ⚙️ Operacional | 3 | Possível necessidade de ajustes técnicos e operacionais nos sistemas que utilizam o DICT. |
+| ⚖️ Regulatório | 2 | Atualização normativa com impacto direto no cumprimento do Regulamento do Pix. |
+| 💰 Financeiro | 1 | Impacto financeiro baixo, limitado a custos de adequação. |
+| 👥 Clientes | 2 | Potencial impacto na experiência do cliente caso ajustes não sejam implementados corretamente. |
 --- Cálculo determinístico ---
 [Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
 [Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
@@ -3527,32 +3527,28 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>bc_-_resolução_bcb_n_573_de_10062026</t>
+          <t>normativos_52923</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>573</t>
+          <t>743</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -3565,98 +3561,201 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I44" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="I44" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K44" s="2" t="inlineStr"/>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc</t>
-        </is>
-      </c>
-      <c r="M44" s="2" t="inlineStr"/>
+          <t>A IN BCB nº 743 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao pix automático, ao pix agendado e ao pix cobrança, para ajustar dispositivos Temas a acompanhar: pagame
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação. | Evidências: liquidação
+[Impacto Financeiro] Score: BAIXO</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Possível necessidade de ajustes nos sistemas e processos relacionados ao Pix Automático. |
+| ⚖️ Regulatório | 4 | Alteração normativa diretamente aplicável ao produto Pix, com impacto em conformidade regulatória. |
+| 💰 Financeiro | 2 | Potencial custo de adequação operacional e risco de penalidades em caso de não conformidade. |
+| 👥 Clientes | 2 | Impacto limitado aos clientes que utilizam Pix Automático, caso haja falhas na implementação. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: ALTO (3/4) | Justificativa: Obrigações regulatórias significativas: liquidação. | Evidências: liquidação
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: MÉDIO (média ponderada: 2.11/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional, Impacto Regulatório. Score médio ponderado: 2.11/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+          <t>Altera a Instrução Normativa BCB nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao Pix Automático, ao Pix Agendado e ao Pix Cobrança, para ajustar dispositivos</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
-        </is>
-      </c>
-      <c r="P44" s="2" t="inlineStr"/>
-      <c r="Q44" s="2" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr"/>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_743_de_11062026</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>743</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="J45" s="4" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 743 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao pix automático, ao pix agendado e ao pix cobrança, para ajustar dispositivos Temas a acompanhar: pagame</t>
+        </is>
+      </c>
       <c r="M45" s="4" t="inlineStr"/>
-      <c r="N45" s="4" t="inlineStr"/>
-      <c r="O45" s="4" t="inlineStr"/>
-      <c r="P45" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Instrução Normativa BCB nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao Pix Automático, ao Pix Agendado e ao Pix Cobrança, para ajustar dispositivos</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="inlineStr"/>
       <c r="Q45" s="4" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_573_de_10062026</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr"/>
-      <c r="O46" s="2" t="inlineStr"/>
-      <c r="P46" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr"/>
       <c r="Q46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr"/>
@@ -3687,7 +3786,7 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
@@ -3695,9 +3794,9 @@
       <c r="D48" s="2" t="inlineStr"/>
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -3718,7 +3817,7 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3726,9 +3825,9 @@
       <c r="D49" s="4" t="inlineStr"/>
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
@@ -3749,7 +3848,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
@@ -3780,7 +3879,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr"/>
@@ -3811,7 +3910,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr"/>
@@ -3819,9 +3918,9 @@
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -3842,7 +3941,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr"/>
@@ -3850,9 +3949,9 @@
       <c r="D53" s="4" t="inlineStr"/>
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
@@ -3873,29 +3972,21 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
@@ -3912,56 +4003,126 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr"/>
       <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F55" s="4" t="inlineStr"/>
       <c r="G55" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H55" s="4" t="inlineStr"/>
       <c r="I55" s="4" t="inlineStr"/>
       <c r="J55" s="4" t="inlineStr"/>
       <c r="K55" s="4" t="inlineStr"/>
       <c r="L55" s="4" t="inlineStr"/>
       <c r="M55" s="4" t="inlineStr"/>
       <c r="N55" s="4" t="inlineStr"/>
-      <c r="O55" s="4" t="inlineStr">
+      <c r="O55" s="4" t="inlineStr"/>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr"/>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr"/>
+      <c r="N57" s="4" t="inlineStr"/>
+      <c r="O57" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P55" s="4" t="inlineStr"/>
-      <c r="Q55" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="inlineStr"/>
+      <c r="Q57" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q55"/>
+  <autoFilter ref="A1:Q57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4034,7 +4195,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4053,11 +4214,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -4080,7 +4241,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4089,7 +4250,7 @@
         </is>
       </c>
       <c r="F5" s="12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -4194,7 +4355,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -4204,13 +4365,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -4286,7 +4447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5916,17 +6077,17 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>573</t>
+          <t>743</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -5934,26 +6095,48 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I43" s="4" t="inlineStr"/>
-      <c r="J43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="n">
+        <v>2.111111111111111</v>
+      </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>743</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
+        </is>
+      </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
@@ -5962,16 +6145,32 @@
       <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr"/>
-      <c r="K44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
+        </is>
+      </c>
       <c r="L44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="4" t="inlineStr"/>
-      <c r="B45" s="4" t="inlineStr"/>
-      <c r="C45" s="4" t="inlineStr"/>
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
@@ -5980,7 +6179,11 @@
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L45" s="4" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
@@ -6022,14 +6225,10 @@
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr"/>
       <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C48" s="2" t="inlineStr"/>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
@@ -6038,15 +6237,55 @@
       <c r="H48" s="2" t="inlineStr"/>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr">
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L48"/>
+  <autoFilter ref="A1:L50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6316,7 +6555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6398,22 +6637,22 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>normativos_52920</t>
+          <t>normativos_52922</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>573</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -6439,7 +6678,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
@@ -6448,7 +6687,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>normativos_52919</t>
+          <t>normativos_52921</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -6458,17 +6697,17 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>740</t>
+          <t>742</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="F3" s="17" t="n">
@@ -6489,7 +6728,7 @@
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr"/>
@@ -6498,7 +6737,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
+          <t>normativos_52920</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -6508,17 +6747,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>739</t>
+          <t>741</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>NÃO APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="F4" s="17" t="n">
@@ -6532,10 +6771,14 @@
           <t>inicial</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
@@ -6544,22 +6787,22 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>normativos_52917</t>
+          <t>normativos_52923</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>572</t>
+          <t>743</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -6580,315 +6823,19 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52921</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>742</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 742 de 09/06/2026</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F6" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52920</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>741</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 741 de 03/06/2026</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52919</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>740</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 740 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="F9" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr"/>
-      <c r="L9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>normativos_52917</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>572</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 572 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-10</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>normativos_52922</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>573</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>inicial</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
-      <c r="L11" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-12 00:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -149,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,6 +200,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -565,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q57"/>
+  <dimension ref="A1:Q59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3621,17 +3622,17 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>bc_-_instrução_normativa_bcb_n_743_de_11062026</t>
+          <t>normativos_52924</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>5.308</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -3639,14 +3640,10 @@
           <t>2026-06-11</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+      <c r="E45" s="4" t="inlineStr"/>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
+          <t>BC - Resolução CMN N° 5.308 de 11/06/2026</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -3656,54 +3653,78 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
-      <c r="I45" s="8" t="inlineStr">
-        <is>
-          <t>MÉDIO</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr"/>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K45" s="4" t="inlineStr"/>
       <c r="L45" s="4" t="inlineStr">
         <is>
-          <t>A IN BCB nº 743 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao pix automático, ao pix agendado e ao pix cobrança, para ajustar dispositivos Temas a acompanhar: pagame</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr"/>
+          <t>A Res. CMN nº 5.308 não é diretamente aplicável mas deve ser monitorada pois dispõe sobre os financiamentos ao amparo de recursos do fundo nacional de investimento em infraestrutura social – fiis para segurança pública. Temas a acompanhar: investimento.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N45" s="4" t="inlineStr">
         <is>
-          <t>Altera a Instrução Normativa BCB nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao Pix Automático, ao Pix Agendado e ao Pix Cobrança, para ajustar dispositivos</t>
+          <t>Dispõe sobre os financiamentos ao amparo de recursos do Fundo Nacional de Investimento em Infraestrutura Social – FIIS para segurança pública.</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743</t>
-        </is>
-      </c>
-      <c r="P45" s="4" t="inlineStr"/>
-      <c r="Q45" s="4" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5308</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>bc_-_resolução_bcb_n_573_de_10062026</t>
+          <t>bc_-_instrução_normativa_bcb_n_743_de_11062026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>573</t>
+          <t>743</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3713,7 +3734,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
@@ -3726,27 +3747,27 @@
           <t>MÉDIA</t>
         </is>
       </c>
-      <c r="I46" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc</t>
+          <t>A IN BCB nº 743 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao pix automático, ao pix agendado e ao pix cobrança, para ajustar dispositivos Temas a acompanhar: pagame</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+          <t>Altera a Instrução Normativa BCB nº 513, de 30 de agosto de 2024, que estabelece os procedimentos operacionais relativos ao Pix Automático, ao Pix Agendado e ao Pix Cobrança, para ajustar dispositivos</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=743</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr"/>
@@ -3755,69 +3776,141 @@
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_573_de_10062026</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J47" s="4" t="inlineStr"/>
       <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 573 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao banco central do brasil relativas à apuração de limites e padrões regulamentares, para incluir  Temas a acompanhar: banc</t>
+        </is>
+      </c>
       <c r="M47" s="4" t="inlineStr"/>
-      <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr"/>
-      <c r="P47" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Altera a Resolução BCB nº 69, de 10 de fevereiro de 2021, que dispõe sobre a prestação de informações ao Banco Central do Brasil relativas à apuração de limites e padrões regulamentares, para incluir </t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=573</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="inlineStr"/>
       <c r="Q47" s="4" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_cmn_n_5308_de_11062026</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>5.308</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.308 de 11/06/2026</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.308 não é diretamente aplicável mas deve ser monitorada pois dispõe sobre os financiamentos ao amparo de recursos do fundo nacional de investimento em infraestrutura social – fiis para segurança pública. Temas a acompanhar: investimento.</t>
+        </is>
+      </c>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr"/>
-      <c r="O48" s="2" t="inlineStr"/>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>Dispõe sobre os financiamentos ao amparo de recursos do Fundo Nacional de Investimento em Infraestrutura Social – FIIS para segurança pública.</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5308](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5308</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr"/>
       <c r="Q48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr"/>
@@ -3848,7 +3941,7 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr"/>
@@ -3856,9 +3949,9 @@
       <c r="D50" s="2" t="inlineStr"/>
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -3879,7 +3972,7 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr"/>
@@ -3887,9 +3980,9 @@
       <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
@@ -3910,7 +4003,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr"/>
@@ -3941,7 +4034,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr"/>
@@ -3972,7 +4065,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
@@ -3980,9 +4073,9 @@
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -4003,7 +4096,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr"/>
@@ -4011,9 +4104,9 @@
       <c r="D55" s="4" t="inlineStr"/>
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
@@ -4034,29 +4127,21 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr"/>
       <c r="C56" s="2" t="inlineStr"/>
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr"/>
@@ -4073,56 +4158,126 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr"/>
+      <c r="C57" s="4" t="inlineStr"/>
+      <c r="D57" s="4" t="inlineStr"/>
       <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F57" s="4" t="inlineStr"/>
       <c r="G57" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H57" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr"/>
       <c r="J57" s="4" t="inlineStr"/>
       <c r="K57" s="4" t="inlineStr"/>
       <c r="L57" s="4" t="inlineStr"/>
       <c r="M57" s="4" t="inlineStr"/>
       <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr">
+      <c r="O57" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr"/>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr"/>
+      <c r="M59" s="4" t="inlineStr"/>
+      <c r="N59" s="4" t="inlineStr"/>
+      <c r="O59" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P57" s="4" t="inlineStr"/>
-      <c r="Q57" s="4" t="inlineStr"/>
+      <c r="P59" s="4" t="inlineStr"/>
+      <c r="Q59" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q57"/>
+  <autoFilter ref="A1:Q59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4195,7 +4350,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4214,11 +4369,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -4260,7 +4415,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7"/>
@@ -4365,13 +4520,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -4379,7 +4534,7 @@
         </is>
       </c>
       <c r="G14" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -4447,7 +4602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6121,17 +6276,17 @@
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução CMN</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>743</t>
+          <t>5.308</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
+          <t>BC - Resolução CMN N° 5.308 de 11/06/2026</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -6139,15 +6294,25 @@
           <t>MONITORAR</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I44" s="2" t="inlineStr"/>
-      <c r="J44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>MÉDIO</t>
+          <t>BAIXO</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr"/>
@@ -6155,17 +6320,17 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>573</t>
+          <t>743</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 743 de 11/06/2026</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -6181,18 +6346,30 @@
       <c r="J45" s="4" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>BAIXO</t>
+          <t>MÉDIO</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="2" t="inlineStr"/>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 573 de 10/06/2026</t>
+        </is>
+      </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
@@ -6201,16 +6378,32 @@
       <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="4" t="inlineStr"/>
-      <c r="B47" s="4" t="inlineStr"/>
-      <c r="C47" s="4" t="inlineStr"/>
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>5.308</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.308 de 11/06/2026</t>
+        </is>
+      </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr"/>
@@ -6219,7 +6412,11 @@
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr"/>
       <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L47" s="4" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -6261,14 +6458,10 @@
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr"/>
       <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
@@ -6277,15 +6470,55 @@
       <c r="H50" s="2" t="inlineStr"/>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr">
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="4" t="inlineStr"/>
+      <c r="B51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr"/>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L50"/>
+  <autoFilter ref="A1:L52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6555,20 +6788,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="43" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -6834,8 +7067,154 @@
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
     </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__740</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB n° 740</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>slack_1780326835.339559_1781001231.942789</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>U097JEJ4KLZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__740</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>740</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB n° 740</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>slack_1780326835.339559_1781035046.419369</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>U05R14K15CH</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52924</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>5.308</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.308 de 11/06/2026</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-13 00:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q59"/>
+  <dimension ref="A1:Q61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3910,69 +3910,168 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr"/>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr"/>
+          <t>normativos_52925</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
       <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr"/>
-      <c r="J49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 744 de 12/06/2026</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>1.222222222222222</v>
+      </c>
       <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="4" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A IN BCB nº 744 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 33, de 29 de outubro de 2020, que estabelece os procedimentos para a remessa das informações de que trata a circular nº 3.979, de 30 de janeiro de 2020, e altera as Temas a acompanhar: risco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: MÉDIO (2/4) | Justificativa: Ajustes pontuais em procedimentos: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] </t>
+        </is>
+      </c>
+      <c r="M49" s="4" t="inlineStr">
+        <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Alterações no leiaute e instruções do DRO podem demandar ajustes em sistemas e processos internos. |
+| ⚖️ Regulatório | 4 | Obrigação regulatória direta de reporte do DRO, com risco de penalidades em caso de não conformidade. |
+| 💰 Financeiro | 2 | Custos moderados para adequação de sistemas e processos, mas sem impacto financeiro direto significativo. |
+| 👥 Clientes | 1 | Sem impacto direto nos clientes. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: MÉDIO (2/4) | Justificativa: Ajustes pontuais em procedimentos: procedimento. | Evidências: procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.22/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.22/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Instrução Normativa BCB nº 33, de 29 de outubro de 2020, que estabelece os procedimentos para a remessa das informações de que trata a Circular nº 3.979, de 30 de janeiro de 2020, e altera as</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=744</t>
+        </is>
+      </c>
       <c r="P49" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q49" s="4" t="inlineStr"/>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="Q49" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_744_de_12062026</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 744 de 12/06/2026</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 744 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 33, de 29 de outubro de 2020, que estabelece os procedimentos para a remessa das informações de que trata a circular nº 3.979, de 30 de janeiro de 2020, e altera as Temas a acompanhar: risco.</t>
+        </is>
+      </c>
       <c r="M50" s="2" t="inlineStr"/>
-      <c r="N50" s="2" t="inlineStr"/>
-      <c r="O50" s="2" t="inlineStr"/>
-      <c r="P50" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Instrução Normativa BCB nº 33, de 29 de outubro de 2020, que estabelece os procedimentos para a remessa das informações de que trata a Circular nº 3.979, de 30 de janeiro de 2020, e altera as</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=744](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=744</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr"/>
       <c r="Q50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr"/>
@@ -4003,7 +4102,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr"/>
@@ -4011,9 +4110,9 @@
       <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
@@ -4034,7 +4133,7 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr"/>
@@ -4042,9 +4141,9 @@
       <c r="D53" s="4" t="inlineStr"/>
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
@@ -4065,7 +4164,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
@@ -4096,7 +4195,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr"/>
@@ -4127,7 +4226,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr"/>
@@ -4135,9 +4234,9 @@
       <c r="D56" s="2" t="inlineStr"/>
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
@@ -4158,7 +4257,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr"/>
@@ -4166,9 +4265,9 @@
       <c r="D57" s="4" t="inlineStr"/>
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
@@ -4189,29 +4288,21 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr"/>
       <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
       <c r="L58" s="2" t="inlineStr"/>
@@ -4228,56 +4319,126 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="4" t="inlineStr"/>
+      <c r="D59" s="4" t="inlineStr"/>
       <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F59" s="4" t="inlineStr"/>
       <c r="G59" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H59" s="4" t="inlineStr"/>
       <c r="I59" s="4" t="inlineStr"/>
       <c r="J59" s="4" t="inlineStr"/>
       <c r="K59" s="4" t="inlineStr"/>
       <c r="L59" s="4" t="inlineStr"/>
       <c r="M59" s="4" t="inlineStr"/>
       <c r="N59" s="4" t="inlineStr"/>
-      <c r="O59" s="4" t="inlineStr">
+      <c r="O59" s="4" t="inlineStr"/>
+      <c r="P59" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr"/>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr"/>
+      <c r="M61" s="4" t="inlineStr"/>
+      <c r="N61" s="4" t="inlineStr"/>
+      <c r="O61" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P59" s="4" t="inlineStr"/>
-      <c r="Q59" s="4" t="inlineStr"/>
+      <c r="P61" s="4" t="inlineStr"/>
+      <c r="Q61" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q59"/>
+  <autoFilter ref="A1:Q61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4350,7 +4511,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4369,11 +4530,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>47%</t>
+          <t>48%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -4415,7 +4576,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7"/>
@@ -4520,13 +4681,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -4534,7 +4695,7 @@
         </is>
       </c>
       <c r="G14" s="13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -4602,7 +4763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6420,30 +6581,68 @@
       <c r="L47" s="4" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 744 de 12/06/2026</t>
+        </is>
+      </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I48" s="2" t="inlineStr"/>
-      <c r="J48" s="2" t="inlineStr"/>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="n">
+        <v>1.222222222222222</v>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="4" t="inlineStr"/>
-      <c r="B49" s="4" t="inlineStr"/>
-      <c r="C49" s="4" t="inlineStr"/>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 744 de 12/06/2026</t>
+        </is>
+      </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr"/>
@@ -6452,7 +6651,11 @@
       <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr"/>
       <c r="J49" s="4" t="inlineStr"/>
-      <c r="K49" s="4" t="inlineStr"/>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L49" s="4" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
@@ -6494,14 +6697,10 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr"/>
       <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
@@ -6510,15 +6709,55 @@
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="4" t="inlineStr"/>
+      <c r="B53" s="4" t="inlineStr"/>
+      <c r="C53" s="4" t="inlineStr"/>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr"/>
+      <c r="K53" s="4" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L52"/>
+  <autoFilter ref="A1:L54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6788,7 +7027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7213,8 +7452,58 @@
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr"/>
     </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52925</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 744 de 12/06/2026</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-15 19:01)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$61</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q61"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4071,69 +4071,161 @@
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr"/>
+          <t>normativos_52926</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
       <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="4" t="inlineStr"/>
-      <c r="J51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 745 de 15/06/2026</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="4" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 745 não é diretamente aplicável mas deve ser monitorada pois institui o plano setorial de prevenção e enfrentamento ao assédio moral, ao assédio sexual e a todas as formas de discriminação do banco central do brasil. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>Institui o Plano Setorial de Prevenção e Enfrentamento ao Assédio Moral, ao Assédio Sexual e a Todas as Formas de Discriminação do Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=745</t>
+        </is>
+      </c>
       <c r="P51" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q51" s="4" t="inlineStr"/>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_745_de_15062026</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 745 de 15/06/2026</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 745 não é diretamente aplicável mas deve ser monitorada pois institui o plano setorial de prevenção e enfrentamento ao assédio moral, ao assédio sexual e a todas as formas de discriminação do banco central do brasil. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
-      <c r="P52" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Institui o Plano Setorial de Prevenção e Enfrentamento ao Assédio Moral, ao Assédio Sexual e a Todas as Formas de Discriminação do Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=745](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=745</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr"/>
       <c r="Q52" s="2" t="inlineStr"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr"/>
@@ -4164,7 +4256,7 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr"/>
@@ -4172,9 +4264,9 @@
       <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -4195,7 +4287,7 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr"/>
@@ -4203,9 +4295,9 @@
       <c r="D55" s="4" t="inlineStr"/>
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
@@ -4226,7 +4318,7 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr"/>
@@ -4257,7 +4349,7 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr"/>
@@ -4288,7 +4380,7 @@
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr"/>
@@ -4296,9 +4388,9 @@
       <c r="D58" s="2" t="inlineStr"/>
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -4319,7 +4411,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr"/>
@@ -4327,9 +4419,9 @@
       <c r="D59" s="4" t="inlineStr"/>
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
@@ -4350,29 +4442,21 @@
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" s="2" t="inlineStr"/>
       <c r="D60" s="2" t="inlineStr"/>
       <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
@@ -4389,56 +4473,126 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr"/>
       <c r="E61" s="4" t="inlineStr"/>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F61" s="4" t="inlineStr"/>
       <c r="G61" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H61" s="4" t="inlineStr"/>
       <c r="I61" s="4" t="inlineStr"/>
       <c r="J61" s="4" t="inlineStr"/>
       <c r="K61" s="4" t="inlineStr"/>
       <c r="L61" s="4" t="inlineStr"/>
       <c r="M61" s="4" t="inlineStr"/>
       <c r="N61" s="4" t="inlineStr"/>
-      <c r="O61" s="4" t="inlineStr">
+      <c r="O61" s="4" t="inlineStr"/>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr"/>
+      <c r="M63" s="4" t="inlineStr"/>
+      <c r="N63" s="4" t="inlineStr"/>
+      <c r="O63" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P61" s="4" t="inlineStr"/>
-      <c r="Q61" s="4" t="inlineStr"/>
+      <c r="P63" s="4" t="inlineStr"/>
+      <c r="Q63" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q61"/>
+  <autoFilter ref="A1:Q63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4511,7 +4665,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4530,11 +4684,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -4557,7 +4711,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4576,7 +4730,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7"/>
@@ -4671,7 +4825,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -4681,13 +4835,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -4763,7 +4917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -6659,30 +6813,68 @@
       <c r="L49" s="4" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="2" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 745 de 15/06/2026</t>
+        </is>
+      </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I50" s="2" t="inlineStr"/>
-      <c r="J50" s="2" t="inlineStr"/>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 745 de 15/06/2026</t>
+        </is>
+      </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr"/>
@@ -6691,7 +6883,11 @@
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr"/>
       <c r="J51" s="4" t="inlineStr"/>
-      <c r="K51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L51" s="4" t="inlineStr"/>
     </row>
     <row r="52" ht="18" customHeight="1">
@@ -6733,14 +6929,10 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr"/>
       <c r="B54" s="2" t="inlineStr"/>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -6749,15 +6941,55 @@
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L54"/>
+  <autoFilter ref="A1:L56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7027,7 +7259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7502,8 +7734,58 @@
       <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="4" t="inlineStr"/>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52926</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 745 de 15/06/2026</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:L10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-17 00:02)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q65"/>
+  <dimension ref="A1:Q71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4312,17 +4312,17 @@
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>bc_-_instrução_normativa_bcb_n_746_de_16062026</t>
+          <t>normativos_52928</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Normativo BCB</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>746</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -4330,14 +4330,10 @@
           <t>2026-06-16</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 746 de 16/06/2026</t>
+          <t>BC - Resolução Coseg N° 2 de 16/06/2026</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -4355,217 +4351,497 @@
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>A IN BCB nº 746 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 512, de 30 de agosto de 2024, que dispõe sobre os limites de valor para as transações no âmbito do pix, para ajustar dispositivos relacionados ao limite de valor qu Temas a acompanhar: pagame</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr"/>
+          <t>A Normativo BCB nº 2 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em belo horizonte. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>Altera a Instrução Normativa BCB nº 512, de 30 de agosto de 2024, que dispõe sobre os limites de valor para as transações no âmbito do Pix, para ajustar dispositivos relacionados ao limite de valor qu</t>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Belo Horizonte.</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=746](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=746</t>
-        </is>
-      </c>
-      <c r="P54" s="2" t="inlineStr"/>
-      <c r="Q54" s="2" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=2</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr"/>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr"/>
+          <t>normativos_52929</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
       <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="4" t="inlineStr"/>
-      <c r="J55" s="4" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 3 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K55" s="4" t="inlineStr"/>
-      <c r="L55" s="4" t="inlineStr"/>
-      <c r="M55" s="4" t="inlineStr"/>
-      <c r="N55" s="4" t="inlineStr"/>
-      <c r="O55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>A Normativo BCB nº 3 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em belém. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Belém.</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=3</t>
+        </is>
+      </c>
       <c r="P55" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q55" s="4" t="inlineStr"/>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr"/>
+          <t>normativos_52930</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
       <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 4 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr"/>
-      <c r="M56" s="2" t="inlineStr"/>
-      <c r="N56" s="2" t="inlineStr"/>
-      <c r="O56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>A Normativo BCB nº 4 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em curitiba. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Curitiba.</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=4</t>
+        </is>
+      </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q56" s="2" t="inlineStr"/>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr"/>
-      <c r="C57" s="4" t="inlineStr"/>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" s="4" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_746_de_16062026</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>746</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 746 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J57" s="4" t="inlineStr"/>
       <c r="K57" s="4" t="inlineStr"/>
-      <c r="L57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 746 não é diretamente aplicável mas deve ser monitorada pois altera a instrução normativa bcb nº 512, de 30 de agosto de 2024, que dispõe sobre os limites de valor para as transações no âmbito do pix, para ajustar dispositivos relacionados ao limite de valor qu Temas a acompanhar: pagame</t>
+        </is>
+      </c>
       <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr"/>
-      <c r="P57" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Instrução Normativa BCB nº 512, de 30 de agosto de 2024, que dispõe sobre os limites de valor para as transações no âmbito do Pix, para ajustar dispositivos relacionados ao limite de valor qu</t>
+        </is>
+      </c>
+      <c r="O57" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=746](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=746</t>
+        </is>
+      </c>
+      <c r="P57" s="4" t="inlineStr"/>
       <c r="Q57" s="4" t="inlineStr"/>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr"/>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_coseg_n_2_de_16062026</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 2 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>A Normativo BCB nº 2 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em belo horizonte. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M58" s="2" t="inlineStr"/>
-      <c r="N58" s="2" t="inlineStr"/>
-      <c r="O58" s="2" t="inlineStr"/>
-      <c r="P58" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Belo Horizonte.</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=2](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=2</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr"/>
       <c r="Q58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr"/>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr"/>
-      <c r="I59" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_coseg_n_3_de_16062026</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 3 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J59" s="4" t="inlineStr"/>
       <c r="K59" s="4" t="inlineStr"/>
-      <c r="L59" s="4" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>A Normativo BCB nº 3 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em belém. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M59" s="4" t="inlineStr"/>
-      <c r="N59" s="4" t="inlineStr"/>
-      <c r="O59" s="4" t="inlineStr"/>
-      <c r="P59" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Belém.</t>
+        </is>
+      </c>
+      <c r="O59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=3](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=3</t>
+        </is>
+      </c>
+      <c r="P59" s="4" t="inlineStr"/>
       <c r="Q59" s="4" t="inlineStr"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr"/>
-      <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_coseg_n_4_de_16062026</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 4 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>A Normativo BCB nº 4 não é diretamente aplicável mas deve ser monitorada pois divulga o regulamento do edifício-sede do banco central do brasil, em curitiba. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr"/>
-      <c r="N60" s="2" t="inlineStr"/>
-      <c r="O60" s="2" t="inlineStr"/>
-      <c r="P60" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>Divulga o Regulamento do Edifício-Sede do Banco Central do Brasil, em Curitiba.</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=4](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20Coseg&amp;numero=4</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr"/>
       <c r="Q60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr"/>
@@ -4573,9 +4849,9 @@
       <c r="D61" s="4" t="inlineStr"/>
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr"/>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G61" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
@@ -4596,7 +4872,7 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr"/>
@@ -4627,7 +4903,7 @@
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr"/>
@@ -4658,29 +4934,21 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr"/>
       <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr"/>
       <c r="L64" s="2" t="inlineStr"/>
@@ -4697,56 +4965,250 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52908</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr"/>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr"/>
       <c r="E65" s="4" t="inlineStr"/>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr"/>
       <c r="I65" s="4" t="inlineStr"/>
       <c r="J65" s="4" t="inlineStr"/>
       <c r="K65" s="4" t="inlineStr"/>
       <c r="L65" s="4" t="inlineStr"/>
       <c r="M65" s="4" t="inlineStr"/>
       <c r="N65" s="4" t="inlineStr"/>
-      <c r="O65" s="4" t="inlineStr">
+      <c r="O65" s="4" t="inlineStr"/>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52907</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52910</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr"/>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr"/>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+      <c r="M67" s="4" t="inlineStr"/>
+      <c r="N67" s="4" t="inlineStr"/>
+      <c r="O67" s="4" t="inlineStr"/>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="C68" s="2" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr"/>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr"/>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr"/>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" s="4" t="inlineStr"/>
+      <c r="O69" s="4" t="inlineStr"/>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr"/>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr"/>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
-      <c r="P65" s="4" t="inlineStr"/>
-      <c r="Q65" s="4" t="inlineStr"/>
+      <c r="P71" s="4" t="inlineStr"/>
+      <c r="Q71" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q65"/>
+  <autoFilter ref="A1:Q71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4819,7 +5281,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -4838,11 +5300,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -4865,7 +5327,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4884,7 +5346,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7"/>
@@ -4979,7 +5441,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -4989,13 +5451,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -5071,7 +5533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -7091,80 +7553,154 @@
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 2 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 3 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 4 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>746</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 746 de 16/06/2026</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr"/>
-      <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="4" t="inlineStr"/>
-      <c r="H53" s="4" t="inlineStr"/>
-      <c r="I53" s="4" t="inlineStr"/>
-      <c r="J53" s="4" t="inlineStr"/>
-      <c r="K53" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="L53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="2" t="inlineStr"/>
-      <c r="B54" s="2" t="inlineStr"/>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
-      <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="4" t="inlineStr"/>
-      <c r="B55" s="4" t="inlineStr"/>
-      <c r="C55" s="4" t="inlineStr"/>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr"/>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="4" t="inlineStr"/>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="4" t="inlineStr"/>
-      <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" s="4" t="inlineStr"/>
-      <c r="L55" s="4" t="inlineStr"/>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="2" t="inlineStr"/>
-      <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr"/>
@@ -7173,16 +7709,32 @@
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
-      <c r="K56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="4" t="inlineStr"/>
-      <c r="B57" s="4" t="inlineStr"/>
-      <c r="C57" s="4" t="inlineStr"/>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 2 de 16/06/2026</t>
+        </is>
+      </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr"/>
@@ -7191,15 +7743,27 @@
       <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr"/>
       <c r="J57" s="4" t="inlineStr"/>
-      <c r="K57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L57" s="4" t="inlineStr"/>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="2" t="inlineStr"/>
-      <c r="B58" s="2" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>BC - Resolução Coseg N° 3 de 16/06/2026</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -7220,8 +7784,140 @@
       </c>
       <c r="L58" s="2" t="inlineStr"/>
     </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 4 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr"/>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="2" t="inlineStr"/>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="4" t="inlineStr"/>
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="4" t="inlineStr"/>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="4" t="inlineStr"/>
+      <c r="B63" s="4" t="inlineStr"/>
+      <c r="C63" s="4" t="inlineStr"/>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="2" t="inlineStr"/>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L58"/>
+  <autoFilter ref="A1:L64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7491,7 +8187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8202,8 +8898,254 @@
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
     </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__745</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>745</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB Nº 745</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>slack_1781550116.095279_1781633031.291959</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>U097D4HTGJY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>instru__o_normativa_bcb_n__744</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>744</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB Nº 744</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>reanalise_feedback</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>slack_1781308899.551779_1781633039.170559</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>U097D4HTGJY</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52930</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 4 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52929</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 3 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52928</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Normativo BCB</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução Coseg N° 2 de 16/06/2026</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L14"/>
+  <autoFilter ref="A1:L19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-17 18:54)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$64</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q71"/>
+  <dimension ref="A1:Q72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5207,8 +5207,59 @@
       <c r="P71" s="4" t="inlineStr"/>
       <c r="Q71" s="4" t="inlineStr"/>
     </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr"/>
+      <c r="N72" s="2" t="inlineStr"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr"/>
+      <c r="Q72" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q71"/>
+  <autoFilter ref="A1:Q72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5281,7 +5332,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -5304,7 +5355,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -5323,11 +5374,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -5417,7 +5468,7 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -5451,7 +5502,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
@@ -7928,7 +7979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8172,8 +8223,46 @@
       </c>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H9"/>
+  <autoFilter ref="A2:H10"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8187,7 +8276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9144,8 +9233,54 @@
       <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr"/>
     </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L19"/>
+  <autoFilter ref="A1:L20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-18 18:55)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$66</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q72"/>
+  <dimension ref="A1:Q74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4841,69 +4841,168 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr"/>
-      <c r="C61" s="4" t="inlineStr"/>
-      <c r="D61" s="4" t="inlineStr"/>
+          <t>normativos_52932</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="E61" s="4" t="inlineStr"/>
-      <c r="F61" s="4" t="inlineStr"/>
-      <c r="G61" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="4" t="inlineStr"/>
-      <c r="J61" s="4" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>1.666666666666667</v>
+      </c>
       <c r="K61" s="4" t="inlineStr"/>
-      <c r="L61" s="4" t="inlineStr"/>
-      <c r="M61" s="4" t="inlineStr"/>
-      <c r="N61" s="4" t="inlineStr"/>
-      <c r="O61" s="4" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 748 não é diretamente aplicável mas deve ser monitorada pois define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no pix na modalidade de provedor de con Temas a acompanhar: capita
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api, procedimento. | Evidências: api, procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Fin</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>| Pilar | Nível | Motivo |
+|---|---|---|
+| ⚙️ Operacional | 3 | Necessidade de monitoramento contínuo e adequação de processos internos. |
+| ⚖️ Regulatório | 4 | Requisito obrigatório para participação no Pix, com impacto direto na conformidade regulatória. |
+| 💰 Financeiro | 3 | Potencial necessidade de recomposição de capital ou patrimônio líquido. |
+| 👥 Clientes | 2 | Impacto indireto, mas relevante para a continuidade das operações no Pix. |
+--- Cálculo determinístico ---
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api, procedimento. | Evidências: api, procedimento
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: MÉDIO (2/4) | Justificativa: Impacto moderado em clientes (não especificado): sac. | Evidências: sac
+Score consolidado: BAIXO (média ponderada: 1.67/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional. Score médio ponderado: 1.67/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>Define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no Pix na modalidade de provedor de con</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748</t>
+        </is>
+      </c>
       <c r="P61" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q61" s="4" t="inlineStr"/>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr"/>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_748_de_18062026</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 748 não é diretamente aplicável mas deve ser monitorada pois define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no pix na modalidade de provedor de con Temas a acompanhar: capita</t>
+        </is>
+      </c>
       <c r="M62" s="2" t="inlineStr"/>
-      <c r="N62" s="2" t="inlineStr"/>
-      <c r="O62" s="2" t="inlineStr"/>
-      <c r="P62" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no Pix na modalidade de provedor de con</t>
+        </is>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr"/>
       <c r="Q62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr"/>
@@ -4934,7 +5033,7 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr"/>
@@ -4942,9 +5041,9 @@
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr"/>
@@ -4965,7 +5064,7 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr"/>
@@ -4973,9 +5072,9 @@
       <c r="D65" s="4" t="inlineStr"/>
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr"/>
-      <c r="G65" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G65" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr"/>
@@ -4996,7 +5095,7 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr"/>
@@ -5027,7 +5126,7 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr"/>
@@ -5058,7 +5157,7 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr"/>
@@ -5066,9 +5165,9 @@
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -5089,7 +5188,7 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr"/>
@@ -5097,9 +5196,9 @@
       <c r="D69" s="4" t="inlineStr"/>
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr"/>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
@@ -5120,29 +5219,21 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr"/>
       <c r="C70" s="2" t="inlineStr"/>
       <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr"/>
@@ -5159,107 +5250,177 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr"/>
+      <c r="C71" s="4" t="inlineStr"/>
+      <c r="D71" s="4" t="inlineStr"/>
       <c r="E71" s="4" t="inlineStr"/>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F71" s="4" t="inlineStr"/>
       <c r="G71" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H71" s="4" t="inlineStr"/>
       <c r="I71" s="4" t="inlineStr"/>
       <c r="J71" s="4" t="inlineStr"/>
       <c r="K71" s="4" t="inlineStr"/>
       <c r="L71" s="4" t="inlineStr"/>
       <c r="M71" s="4" t="inlineStr"/>
       <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
-        </is>
-      </c>
-      <c r="P71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr"/>
+      <c r="P71" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q71" s="4" t="inlineStr"/>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>normativos_52931</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>747</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
-        </is>
-      </c>
-      <c r="G72" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr"/>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr"/>
       <c r="N72" s="2" t="inlineStr"/>
-      <c r="O72" s="2" t="inlineStr">
+      <c r="O72" s="2" t="inlineStr"/>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr"/>
+      <c r="J73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+      <c r="M73" s="4" t="inlineStr"/>
+      <c r="N73" s="4" t="inlineStr"/>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
+        </is>
+      </c>
+      <c r="P73" s="4" t="inlineStr"/>
+      <c r="Q73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
         </is>
       </c>
-      <c r="P72" s="2" t="inlineStr"/>
-      <c r="Q72" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr"/>
+      <c r="Q74" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q72"/>
+  <autoFilter ref="A1:Q74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5351,11 +5512,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -5397,7 +5558,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7"/>
@@ -5492,7 +5653,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
@@ -5502,13 +5663,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -5584,7 +5745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -7870,30 +8031,68 @@
       <c r="L59" s="4" t="inlineStr"/>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="2" t="inlineStr"/>
-      <c r="B60" s="2" t="inlineStr"/>
-      <c r="C60" s="2" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr"/>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="n">
+        <v>1.666666666666667</v>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="4" t="inlineStr"/>
-      <c r="B61" s="4" t="inlineStr"/>
-      <c r="C61" s="4" t="inlineStr"/>
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr"/>
@@ -7902,7 +8101,11 @@
       <c r="H61" s="4" t="inlineStr"/>
       <c r="I61" s="4" t="inlineStr"/>
       <c r="J61" s="4" t="inlineStr"/>
-      <c r="K61" s="4" t="inlineStr"/>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L61" s="4" t="inlineStr"/>
     </row>
     <row r="62" ht="18" customHeight="1">
@@ -7944,14 +8147,10 @@
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr"/>
       <c r="B64" s="2" t="inlineStr"/>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr"/>
@@ -7960,15 +8159,55 @@
       <c r="H64" s="2" t="inlineStr"/>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="4" t="inlineStr"/>
+      <c r="B65" s="4" t="inlineStr"/>
+      <c r="C65" s="4" t="inlineStr"/>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr"/>
+      <c r="J65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="2" t="inlineStr"/>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L64"/>
+  <autoFilter ref="A1:L66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8276,7 +8515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9279,8 +9518,58 @@
       <c r="K20" s="2" t="inlineStr"/>
       <c r="L20" s="2" t="inlineStr"/>
     </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52932</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L20"/>
+  <autoFilter ref="A1:L21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-19 00:05)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q74"/>
+  <dimension ref="A1:Q77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4935,17 +4935,17 @@
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>bc_-_instrução_normativa_bcb_n_748_de_18062026</t>
+          <t>normativos_52934</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>748</t>
+          <t>575</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -4953,14 +4953,10 @@
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Verificar texto integral</t>
-        </is>
-      </c>
+      <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+          <t>BC - Resolução BCB N° 575 de 18/06/2026</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -4978,93 +4974,189 @@
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="n">
+        <v>1.777777777777778</v>
+      </c>
       <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>A IN BCB nº 748 não é diretamente aplicável mas deve ser monitorada pois define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no pix na modalidade de provedor de con Temas a acompanhar: capita</t>
-        </is>
-      </c>
-      <c r="M62" s="2" t="inlineStr"/>
+          <t>A Res. BCB nº 575 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 277, de 31 de dezembro de 2022, e a resolução bcb nº 278, de 31 de dezembro de 2022, para dispor sobre contas de depósito em moeda estrangeira tituladas por pessoas jurídicas Temas a acompanhar: depó
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api. | Evidências: api
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve. | Evidências: deve
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impact</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: api. | Evidências: api
+[Impacto Regulatório] Score: MÉDIO (2/4) | Justificativa: Obrigações regulatórias identificadas: deve. | Evidências: deve
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.78/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional. Score médio ponderado: 1.78/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>Define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no Pix na modalidade de provedor de con</t>
+          <t>Altera a Resolução BCB nº 277, de 31 de dezembro de 2022, e a Resolução BCB nº 278, de 31 de dezembro de 2022, para dispor sobre contas de depósito em moeda estrangeira tituladas por pessoas jurídicas</t>
         </is>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748</t>
-        </is>
-      </c>
-      <c r="P62" s="2" t="inlineStr"/>
-      <c r="Q62" s="2" t="inlineStr"/>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=575</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr"/>
-      <c r="C63" s="4" t="inlineStr"/>
-      <c r="D63" s="4" t="inlineStr"/>
-      <c r="E63" s="4" t="inlineStr"/>
-      <c r="F63" s="4" t="inlineStr"/>
-      <c r="G63" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="4" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_748_de_18062026</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J63" s="4" t="inlineStr"/>
       <c r="K63" s="4" t="inlineStr"/>
-      <c r="L63" s="4" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 748 não é diretamente aplicável mas deve ser monitorada pois define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no pix na modalidade de provedor de con Temas a acompanhar: capita</t>
+        </is>
+      </c>
       <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" s="4" t="inlineStr"/>
-      <c r="O63" s="4" t="inlineStr"/>
-      <c r="P63" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>Define os procedimentos para a verificação do cumprimento dos limites mínimos de capital social integralizado e de patrimônio líquido, para fins de participação no Pix na modalidade de provedor de con</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=748</t>
+        </is>
+      </c>
+      <c r="P63" s="4" t="inlineStr"/>
       <c r="Q63" s="4" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr"/>
-      <c r="C64" s="2" t="inlineStr"/>
-      <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_575_de_18062026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 575 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 575 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 277, de 31 de dezembro de 2022, e a resolução bcb nº 278, de 31 de dezembro de 2022, para dispor sobre contas de depósito em moeda estrangeira tituladas por pessoas jurídicas Temas a acompanhar: depó</t>
+        </is>
+      </c>
       <c r="M64" s="2" t="inlineStr"/>
-      <c r="N64" s="2" t="inlineStr"/>
-      <c r="O64" s="2" t="inlineStr"/>
-      <c r="P64" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Resolução BCB nº 277, de 31 de dezembro de 2022, e a Resolução BCB nº 278, de 31 de dezembro de 2022, para dispor sobre contas de depósito em moeda estrangeira tituladas por pessoas jurídicas</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=575](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=575</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr"/>
       <c r="Q64" s="2" t="inlineStr"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr"/>
@@ -5095,7 +5187,7 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr"/>
@@ -5103,9 +5195,9 @@
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -5126,7 +5218,7 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr"/>
@@ -5134,9 +5226,9 @@
       <c r="D67" s="4" t="inlineStr"/>
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr"/>
@@ -5157,7 +5249,7 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr"/>
@@ -5188,7 +5280,7 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr"/>
@@ -5219,7 +5311,7 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr"/>
@@ -5227,9 +5319,9 @@
       <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
@@ -5250,7 +5342,7 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr"/>
@@ -5258,9 +5350,9 @@
       <c r="D71" s="4" t="inlineStr"/>
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr"/>
-      <c r="G71" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
@@ -5281,29 +5373,21 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr"/>
       <c r="C72" s="2" t="inlineStr"/>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr"/>
@@ -5320,107 +5404,228 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr"/>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr"/>
       <c r="E73" s="4" t="inlineStr"/>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F73" s="4" t="inlineStr"/>
       <c r="G73" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H73" s="4" t="inlineStr"/>
       <c r="I73" s="4" t="inlineStr"/>
       <c r="J73" s="4" t="inlineStr"/>
       <c r="K73" s="4" t="inlineStr"/>
       <c r="L73" s="4" t="inlineStr"/>
       <c r="M73" s="4" t="inlineStr"/>
       <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
-        </is>
-      </c>
-      <c r="P73" s="4" t="inlineStr"/>
+      <c r="O73" s="4" t="inlineStr"/>
+      <c r="P73" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q73" s="4" t="inlineStr"/>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>normativos_52931</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>747</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
-        </is>
-      </c>
-      <c r="G74" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr"/>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
       <c r="M74" s="2" t="inlineStr"/>
       <c r="N74" s="2" t="inlineStr"/>
-      <c r="O74" s="2" t="inlineStr">
+      <c r="O74" s="2" t="inlineStr"/>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G75" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr"/>
+      <c r="N75" s="4" t="inlineStr"/>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
+        </is>
+      </c>
+      <c r="P75" s="4" t="inlineStr"/>
+      <c r="Q75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr"/>
+      <c r="O76" s="2" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
         </is>
       </c>
-      <c r="P74" s="2" t="inlineStr"/>
-      <c r="Q74" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr"/>
+      <c r="Q76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52933</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr"/>
+      <c r="J77" s="4" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+      <c r="M77" s="4" t="inlineStr"/>
+      <c r="N77" s="4" t="inlineStr"/>
+      <c r="O77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
+        </is>
+      </c>
+      <c r="P77" s="4" t="inlineStr"/>
+      <c r="Q77" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q74"/>
+  <autoFilter ref="A1:Q77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5493,7 +5698,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -5512,11 +5717,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -5535,11 +5740,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -5558,7 +5763,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7"/>
@@ -5629,7 +5834,7 @@
         </is>
       </c>
       <c r="G12" s="13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -5653,7 +5858,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
@@ -5663,13 +5868,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -5745,7 +5950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8077,44 +8282,66 @@
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 575 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="n">
+        <v>1.777777777777778</v>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>Instrução Normativa BCB</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>748</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>BC - Instrução Normativa BCB N° 748 de 18/06/2026</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>MONITORAR</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr"/>
-      <c r="F61" s="4" t="inlineStr"/>
-      <c r="G61" s="4" t="inlineStr"/>
-      <c r="H61" s="4" t="inlineStr"/>
-      <c r="I61" s="4" t="inlineStr"/>
-      <c r="J61" s="4" t="inlineStr"/>
-      <c r="K61" s="4" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
-      <c r="L61" s="4" t="inlineStr"/>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="2" t="inlineStr"/>
-      <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr"/>
@@ -8123,16 +8350,32 @@
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="4" t="inlineStr"/>
-      <c r="B63" s="4" t="inlineStr"/>
-      <c r="C63" s="4" t="inlineStr"/>
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 575 de 18/06/2026</t>
+        </is>
+      </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr"/>
@@ -8141,7 +8384,11 @@
       <c r="H63" s="4" t="inlineStr"/>
       <c r="I63" s="4" t="inlineStr"/>
       <c r="J63" s="4" t="inlineStr"/>
-      <c r="K63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L63" s="4" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
@@ -8183,14 +8430,10 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="2" t="inlineStr"/>
       <c r="B66" s="2" t="inlineStr"/>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C66" s="2" t="inlineStr"/>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr"/>
@@ -8199,15 +8442,55 @@
       <c r="H66" s="2" t="inlineStr"/>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr"/>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr"/>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="2" t="inlineStr"/>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L66"/>
+  <autoFilter ref="A1:L68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8218,7 +8501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8500,8 +8783,46 @@
       </c>
       <c r="H10" s="16" t="inlineStr"/>
     </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52933</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H10"/>
+  <autoFilter ref="A2:H11"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8515,7 +8836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9568,8 +9889,104 @@
       <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="4" t="inlineStr"/>
     </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52934</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 575 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52933</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L21"/>
+  <autoFilter ref="A1:L23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-19 18:55)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q77"/>
+  <dimension ref="A1:Q78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5624,8 +5624,59 @@
       <c r="P77" s="4" t="inlineStr"/>
       <c r="Q77" s="4" t="inlineStr"/>
     </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr"/>
+      <c r="Q78" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q77"/>
+  <autoFilter ref="A1:Q78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5721,7 +5772,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -5740,11 +5791,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -5858,7 +5909,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14">
@@ -5868,7 +5919,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
@@ -8501,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8821,8 +8872,46 @@
       </c>
       <c r="H11" s="4" t="inlineStr"/>
     </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H11"/>
+  <autoFilter ref="A2:H12"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8836,7 +8925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9985,8 +10074,54 @@
       <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="4" t="inlineStr"/>
     </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
+  <autoFilter ref="A1:L24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-20 00:04)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$68</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q78"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5156,69 +5156,161 @@
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr"/>
-      <c r="C65" s="4" t="inlineStr"/>
-      <c r="D65" s="4" t="inlineStr"/>
+          <t>normativos_52937</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>5.309</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
       <c r="E65" s="4" t="inlineStr"/>
-      <c r="F65" s="4" t="inlineStr"/>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="4" t="inlineStr"/>
-      <c r="J65" s="4" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.309 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>1.222222222222222</v>
+      </c>
       <c r="K65" s="4" t="inlineStr"/>
-      <c r="L65" s="4" t="inlineStr"/>
-      <c r="M65" s="4" t="inlineStr"/>
-      <c r="N65" s="4" t="inlineStr"/>
-      <c r="O65" s="4" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.309 não é diretamente aplicável mas deve ser monitorada pois estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para investimentos de que trata o art. 8º-a da lei nº 14.947, de 2 Temas a acompanhar: in
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M65" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: MÉDIO (2/4) | Justificativa: Impacto financeiro moderado: encargo. | Evidências: encargo
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.22/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.22/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para investimentos de que trata o art. 8º-A da Lei nº 14.947, de 2</t>
+        </is>
+      </c>
+      <c r="O65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5309</t>
+        </is>
+      </c>
       <c r="P65" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q65" s="4" t="inlineStr"/>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="Q65" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_cmn_n_5309_de_19062026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>5.309</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.309 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>A Res. CMN nº 5.309 não é diretamente aplicável mas deve ser monitorada pois estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para investimentos de que trata o art. 8º-a da lei nº 14.947, de 2 Temas a acompanhar: in</t>
+        </is>
+      </c>
       <c r="M66" s="2" t="inlineStr"/>
-      <c r="N66" s="2" t="inlineStr"/>
-      <c r="O66" s="2" t="inlineStr"/>
-      <c r="P66" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>Estabelece as condições, os encargos financeiros, os prazos e as demais normas regulamentadoras aplicáveis às linhas de financiamento para investimentos de que trata o art. 8º-A da Lei nº 14.947, de 2</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5309](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20CMN&amp;numero=5309</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr"/>
       <c r="Q66" s="2" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr"/>
@@ -5249,7 +5341,7 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr"/>
@@ -5257,9 +5349,9 @@
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -5280,7 +5372,7 @@
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr"/>
@@ -5288,9 +5380,9 @@
       <c r="D69" s="4" t="inlineStr"/>
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr"/>
-      <c r="G69" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
@@ -5311,7 +5403,7 @@
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr"/>
@@ -5342,7 +5434,7 @@
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr"/>
@@ -5373,7 +5465,7 @@
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr"/>
@@ -5381,9 +5473,9 @@
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -5404,7 +5496,7 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr"/>
@@ -5412,9 +5504,9 @@
       <c r="D73" s="4" t="inlineStr"/>
       <c r="E73" s="4" t="inlineStr"/>
       <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
@@ -5435,29 +5527,21 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G74" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr"/>
@@ -5474,130 +5558,98 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr"/>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr"/>
       <c r="E75" s="4" t="inlineStr"/>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F75" s="4" t="inlineStr"/>
       <c r="G75" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H75" s="4" t="inlineStr"/>
       <c r="I75" s="4" t="inlineStr"/>
       <c r="J75" s="4" t="inlineStr"/>
       <c r="K75" s="4" t="inlineStr"/>
       <c r="L75" s="4" t="inlineStr"/>
       <c r="M75" s="4" t="inlineStr"/>
       <c r="N75" s="4" t="inlineStr"/>
-      <c r="O75" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
-        </is>
-      </c>
-      <c r="P75" s="4" t="inlineStr"/>
+      <c r="O75" s="4" t="inlineStr"/>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q75" s="4" t="inlineStr"/>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>normativos_52931</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>747</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
-        </is>
-      </c>
-      <c r="G76" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr"/>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
       <c r="M76" s="2" t="inlineStr"/>
       <c r="N76" s="2" t="inlineStr"/>
-      <c r="O76" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
-        </is>
-      </c>
-      <c r="P76" s="2" t="inlineStr"/>
+      <c r="O76" s="2" t="inlineStr"/>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q76" s="2" t="inlineStr"/>
     </row>
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>normativos_52933</t>
+          <t>normativos_52918</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>739</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
@@ -5618,7 +5670,7 @@
       <c r="N77" s="4" t="inlineStr"/>
       <c r="O77" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
       <c r="P77" s="4" t="inlineStr"/>
@@ -5627,7 +5679,7 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>normativos_52935</t>
+          <t>normativos_52931</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -5637,18 +5689,18 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>747</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
         </is>
       </c>
       <c r="G78" s="9" t="inlineStr">
@@ -5658,7 +5710,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -5669,14 +5721,167 @@
       <c r="N78" s="2" t="inlineStr"/>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr"/>
       <c r="Q78" s="2" t="inlineStr"/>
     </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52933</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr"/>
+      <c r="J79" s="4" t="inlineStr"/>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+      <c r="M79" s="4" t="inlineStr"/>
+      <c r="N79" s="4" t="inlineStr"/>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="inlineStr"/>
+      <c r="Q79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr"/>
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="inlineStr"/>
+      <c r="Q80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52936</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr"/>
+      <c r="J81" s="4" t="inlineStr"/>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+      <c r="M81" s="4" t="inlineStr"/>
+      <c r="N81" s="4" t="inlineStr"/>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=750</t>
+        </is>
+      </c>
+      <c r="P81" s="4" t="inlineStr"/>
+      <c r="Q81" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q78"/>
+  <autoFilter ref="A1:Q81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5749,7 +5954,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -5768,7 +5973,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
@@ -5791,11 +5996,11 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -5814,7 +6019,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7"/>
@@ -5909,7 +6114,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14">
@@ -5919,13 +6124,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -5933,7 +6138,7 @@
         </is>
       </c>
       <c r="G14" s="13" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -6001,7 +6206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8443,30 +8648,68 @@
       <c r="L63" s="4" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="2" t="inlineStr"/>
-      <c r="B64" s="2" t="inlineStr"/>
-      <c r="C64" s="2" t="inlineStr"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>5.309</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.309 de 19/06/2026</t>
+        </is>
+      </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I64" s="2" t="inlineStr"/>
-      <c r="J64" s="2" t="inlineStr"/>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="n">
+        <v>1.222222222222222</v>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L64" s="2" t="inlineStr"/>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="4" t="inlineStr"/>
-      <c r="B65" s="4" t="inlineStr"/>
-      <c r="C65" s="4" t="inlineStr"/>
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>5.309</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.309 de 19/06/2026</t>
+        </is>
+      </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr"/>
@@ -8475,7 +8718,11 @@
       <c r="H65" s="4" t="inlineStr"/>
       <c r="I65" s="4" t="inlineStr"/>
       <c r="J65" s="4" t="inlineStr"/>
-      <c r="K65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L65" s="4" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
@@ -8517,14 +8764,10 @@
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr"/>
       <c r="B68" s="2" t="inlineStr"/>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C68" s="2" t="inlineStr"/>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr"/>
@@ -8533,15 +8776,55 @@
       <c r="H68" s="2" t="inlineStr"/>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr"/>
-      <c r="K68" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="4" t="inlineStr"/>
+      <c r="B69" s="4" t="inlineStr"/>
+      <c r="C69" s="4" t="inlineStr"/>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="2" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr"/>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L68"/>
+  <autoFilter ref="A1:L70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8552,7 +8835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -8910,8 +9193,46 @@
       </c>
       <c r="H12" s="16" t="inlineStr"/>
     </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52936</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Tema fora do escopo do iFood Pago</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H12"/>
+  <autoFilter ref="A2:H13"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -8925,7 +9246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -10120,8 +10441,104 @@
       <c r="K24" s="2" t="inlineStr"/>
       <c r="L24" s="2" t="inlineStr"/>
     </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52937</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Resolução CMN</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>5.309</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução CMN N° 5.309 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52936</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L24"/>
+  <autoFilter ref="A1:L26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-24 00:05)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q81"/>
+  <dimension ref="A1:Q87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5310,193 +5310,469 @@
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr"/>
-      <c r="C67" s="4" t="inlineStr"/>
-      <c r="D67" s="4" t="inlineStr"/>
+          <t>normativos_52938</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="E67" s="4" t="inlineStr"/>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr"/>
-      <c r="I67" s="4" t="inlineStr"/>
-      <c r="J67" s="4" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 576 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K67" s="4" t="inlineStr"/>
-      <c r="L67" s="4" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" s="4" t="inlineStr"/>
-      <c r="O67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 576 aplica-se diretamente ao iFood Pago pois dispõe sobre a política de sucessão de administradores das administradoras de consórcio, das sociedades corretoras de títulos e valores mobiliários, das sociedades distribuidoras de títulos e valores  Menciona explicitamente: instituições de
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispõe sobre a política de sucessão de administradores das administradoras de consórcio, das sociedades corretoras de títulos e valores mobiliários, das sociedades distribuidoras de títulos e valores </t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=576</t>
+        </is>
+      </c>
       <c r="P67" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q67" s="4" t="inlineStr"/>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr"/>
-      <c r="C68" s="2" t="inlineStr"/>
-      <c r="D68" s="2" t="inlineStr"/>
+          <t>normativos_52939</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 577 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>1.444444444444444</v>
+      </c>
       <c r="K68" s="2" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr"/>
-      <c r="M68" s="2" t="inlineStr"/>
-      <c r="N68" s="2" t="inlineStr"/>
-      <c r="O68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 577 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 207, de 22 de março de 2022, que consolida e altera atos normativos referentes à remessa de informações sobre o controle da exposição ao risco de liquidez e sobre o indicador Temas a acompanhar: liqu
+### Avaliação de Risco:
+[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: controle. | Evidências: controle
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BA</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: ALTO (3/4) | Justificativa: Impacto em processos operacionais: controle. | Evidências: controle
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.44/4.0, divisor 4.5)
+Lógica: Pilares ALTOS: Impacto Operacional. Score médio ponderado: 1.44/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>Altera a Resolução BCB nº 207, de 22 de março de 2022, que consolida e altera atos normativos referentes à remessa de informações sobre o controle da exposição ao risco de liquidez e sobre o indicador</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=577</t>
+        </is>
+      </c>
       <c r="P68" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q68" s="2" t="inlineStr"/>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr"/>
-      <c r="C69" s="4" t="inlineStr"/>
-      <c r="D69" s="4" t="inlineStr"/>
+          <t>normativos_52940</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="E69" s="4" t="inlineStr"/>
-      <c r="F69" s="4" t="inlineStr"/>
-      <c r="G69" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="4" t="inlineStr"/>
-      <c r="J69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 578 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K69" s="4" t="inlineStr"/>
-      <c r="L69" s="4" t="inlineStr"/>
-      <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" s="4" t="inlineStr"/>
-      <c r="O69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 578 não é diretamente aplicável mas deve ser monitorada pois divulga alterações no regimento interno do banco central do brasil. Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M69" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N69" s="4" t="inlineStr">
+        <is>
+          <t>Divulga alterações no Regimento Interno do Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O69" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=578</t>
+        </is>
+      </c>
       <c r="P69" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q69" s="4" t="inlineStr"/>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr"/>
-      <c r="C70" s="2" t="inlineStr"/>
-      <c r="D70" s="2" t="inlineStr"/>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_576_de_23062026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 576 de 23/06/2026</t>
+        </is>
+      </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
-      <c r="L70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 576 aplica-se diretamente ao iFood Pago pois dispõe sobre a política de sucessão de administradores das administradoras de consórcio, das sociedades corretoras de títulos e valores mobiliários, das sociedades distribuidoras de títulos e valores  Menciona explicitamente: instituições de</t>
+        </is>
+      </c>
       <c r="M70" s="2" t="inlineStr"/>
-      <c r="N70" s="2" t="inlineStr"/>
-      <c r="O70" s="2" t="inlineStr"/>
-      <c r="P70" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispõe sobre a política de sucessão de administradores das administradoras de consórcio, das sociedades corretoras de títulos e valores mobiliários, das sociedades distribuidoras de títulos e valores </t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=576](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=576</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr"/>
       <c r="Q70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr"/>
-      <c r="C71" s="4" t="inlineStr"/>
-      <c r="D71" s="4" t="inlineStr"/>
-      <c r="E71" s="4" t="inlineStr"/>
-      <c r="F71" s="4" t="inlineStr"/>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="4" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_577_de_23062026</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 577 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>BAIXA</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J71" s="4" t="inlineStr"/>
       <c r="K71" s="4" t="inlineStr"/>
-      <c r="L71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 577 não é diretamente aplicável mas deve ser monitorada pois altera a resolução bcb nº 207, de 22 de março de 2022, que consolida e altera atos normativos referentes à remessa de informações sobre o controle da exposição ao risco de liquidez e sobre o indicador Temas a acompanhar: liqu</t>
+        </is>
+      </c>
       <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
-      <c r="P71" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N71" s="4" t="inlineStr">
+        <is>
+          <t>Altera a Resolução BCB nº 207, de 22 de março de 2022, que consolida e altera atos normativos referentes à remessa de informações sobre o controle da exposição ao risco de liquidez e sobre o indicador</t>
+        </is>
+      </c>
+      <c r="O71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=577](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=577</t>
+        </is>
+      </c>
+      <c r="P71" s="4" t="inlineStr"/>
       <c r="Q71" s="4" t="inlineStr"/>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr"/>
-      <c r="C72" s="2" t="inlineStr"/>
-      <c r="D72" s="2" t="inlineStr"/>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
+          <t>bc_-_resolução_bcb_n_578_de_23062026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 578 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
-      <c r="L72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>A Res. BCB nº 578 não é diretamente aplicável mas deve ser monitorada pois divulga alterações no regimento interno do banco central do brasil. Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M72" s="2" t="inlineStr"/>
-      <c r="N72" s="2" t="inlineStr"/>
-      <c r="O72" s="2" t="inlineStr"/>
-      <c r="P72" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Divulga alterações no Regimento Interno do Banco Central do Brasil.</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=578](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=578</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr"/>
       <c r="Q72" s="2" t="inlineStr"/>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr"/>
@@ -5504,9 +5780,9 @@
       <c r="D73" s="4" t="inlineStr"/>
       <c r="E73" s="4" t="inlineStr"/>
       <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G73" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
@@ -5527,7 +5803,7 @@
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr"/>
@@ -5558,7 +5834,7 @@
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr"/>
@@ -5589,29 +5865,21 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr"/>
@@ -5628,260 +5896,454 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52908</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr"/>
+      <c r="C77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr"/>
       <c r="E77" s="4" t="inlineStr"/>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
-      <c r="G77" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr"/>
       <c r="I77" s="4" t="inlineStr"/>
       <c r="J77" s="4" t="inlineStr"/>
       <c r="K77" s="4" t="inlineStr"/>
       <c r="L77" s="4" t="inlineStr"/>
       <c r="M77" s="4" t="inlineStr"/>
       <c r="N77" s="4" t="inlineStr"/>
-      <c r="O77" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
-        </is>
-      </c>
-      <c r="P77" s="4" t="inlineStr"/>
+      <c r="O77" s="4" t="inlineStr"/>
+      <c r="P77" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q77" s="4" t="inlineStr"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>normativos_52931</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>747</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+          <t>normativos_52907</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
       <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
-        </is>
-      </c>
-      <c r="G78" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr"/>
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr"/>
       <c r="L78" s="2" t="inlineStr"/>
       <c r="M78" s="2" t="inlineStr"/>
       <c r="N78" s="2" t="inlineStr"/>
-      <c r="O78" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
-        </is>
-      </c>
-      <c r="P78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr"/>
+      <c r="P78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q78" s="2" t="inlineStr"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>normativos_52933</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>Resolução BCB</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>574</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+          <t>normativos_52910</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr"/>
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr"/>
       <c r="E79" s="4" t="inlineStr"/>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
-        </is>
-      </c>
-      <c r="G79" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr"/>
       <c r="I79" s="4" t="inlineStr"/>
       <c r="J79" s="4" t="inlineStr"/>
       <c r="K79" s="4" t="inlineStr"/>
       <c r="L79" s="4" t="inlineStr"/>
       <c r="M79" s="4" t="inlineStr"/>
       <c r="N79" s="4" t="inlineStr"/>
-      <c r="O79" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
-        </is>
-      </c>
-      <c r="P79" s="4" t="inlineStr"/>
+      <c r="O79" s="4" t="inlineStr"/>
+      <c r="P79" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q79" s="4" t="inlineStr"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>normativos_52935</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>749</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+          <t>normativos_52906</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr"/>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
-        </is>
-      </c>
+      <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
+      <c r="H80" s="2" t="inlineStr"/>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr"/>
       <c r="L80" s="2" t="inlineStr"/>
       <c r="M80" s="2" t="inlineStr"/>
       <c r="N80" s="2" t="inlineStr"/>
-      <c r="O80" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
-        </is>
-      </c>
-      <c r="P80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q80" s="2" t="inlineStr"/>
     </row>
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>normativos_52936</t>
-        </is>
-      </c>
-      <c r="B81" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr">
-        <is>
-          <t>750</t>
-        </is>
-      </c>
-      <c r="D81" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr"/>
+      <c r="C81" s="4" t="inlineStr"/>
+      <c r="D81" s="4" t="inlineStr"/>
       <c r="E81" s="4" t="inlineStr"/>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
-        </is>
-      </c>
+      <c r="F81" s="4" t="inlineStr"/>
       <c r="G81" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H81" s="4" t="inlineStr">
-        <is>
-          <t>MÉDIA</t>
-        </is>
-      </c>
+      <c r="H81" s="4" t="inlineStr"/>
       <c r="I81" s="4" t="inlineStr"/>
       <c r="J81" s="4" t="inlineStr"/>
       <c r="K81" s="4" t="inlineStr"/>
       <c r="L81" s="4" t="inlineStr"/>
       <c r="M81" s="4" t="inlineStr"/>
       <c r="N81" s="4" t="inlineStr"/>
-      <c r="O81" s="4" t="inlineStr">
+      <c r="O81" s="4" t="inlineStr"/>
+      <c r="P81" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr"/>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="inlineStr"/>
+      <c r="O82" s="2" t="inlineStr"/>
+      <c r="P82" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="Q82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52918</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
+        </is>
+      </c>
+      <c r="G83" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr"/>
+      <c r="J83" s="4" t="inlineStr"/>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+      <c r="M83" s="4" t="inlineStr"/>
+      <c r="N83" s="4" t="inlineStr"/>
+      <c r="O83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
+        </is>
+      </c>
+      <c r="P83" s="4" t="inlineStr"/>
+      <c r="Q83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52931</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>747</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
+        </is>
+      </c>
+      <c r="G84" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr"/>
+      <c r="Q84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52933</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+        </is>
+      </c>
+      <c r="G85" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr"/>
+      <c r="J85" s="4" t="inlineStr"/>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="4" t="inlineStr"/>
+      <c r="N85" s="4" t="inlineStr"/>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="inlineStr"/>
+      <c r="Q85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G86" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr"/>
+      <c r="Q86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52936</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="4" t="inlineStr"/>
+      <c r="N87" s="4" t="inlineStr"/>
+      <c r="O87" s="4" t="inlineStr">
         <is>
           <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=750</t>
         </is>
       </c>
-      <c r="P81" s="4" t="inlineStr"/>
-      <c r="Q81" s="4" t="inlineStr"/>
+      <c r="P87" s="4" t="inlineStr"/>
+      <c r="Q87" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q81"/>
+  <autoFilter ref="A1:Q87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5950,7 +6412,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
@@ -5973,11 +6435,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>56%</t>
+          <t>57%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -6000,7 +6462,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -6019,7 +6481,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7"/>
@@ -6114,7 +6576,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
@@ -6124,21 +6586,21 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="13" t="n">
         <v>32</v>
       </c>
-      <c r="C14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>28</v>
-      </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
           <t>BAIXA</t>
         </is>
       </c>
       <c r="G14" s="13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -6206,7 +6668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -8726,63 +9188,153 @@
       <c r="L65" s="4" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="2" t="inlineStr"/>
-      <c r="B66" s="2" t="inlineStr"/>
-      <c r="C66" s="2" t="inlineStr"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 576 de 23/06/2026</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I66" s="2" t="inlineStr"/>
-      <c r="J66" s="2" t="inlineStr"/>
-      <c r="K66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L66" s="2" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="4" t="inlineStr"/>
-      <c r="B67" s="4" t="inlineStr"/>
-      <c r="C67" s="4" t="inlineStr"/>
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 577 de 23/06/2026</t>
+        </is>
+      </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr"/>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="4" t="inlineStr"/>
-      <c r="H67" s="4" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I67" s="4" t="inlineStr"/>
-      <c r="J67" s="4" t="inlineStr"/>
-      <c r="K67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="n">
+        <v>1.444444444444444</v>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L67" s="4" t="inlineStr"/>
     </row>
     <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="2" t="inlineStr"/>
-      <c r="B68" s="2" t="inlineStr"/>
-      <c r="C68" s="2" t="inlineStr"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 578 de 23/06/2026</t>
+        </is>
+      </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-      <c r="K68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L68" s="2" t="inlineStr"/>
     </row>
     <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="4" t="inlineStr"/>
-      <c r="B69" s="4" t="inlineStr"/>
-      <c r="C69" s="4" t="inlineStr"/>
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 576 de 23/06/2026</t>
+        </is>
+      </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
           <t>APLICÁVEL</t>
@@ -8794,15 +9346,27 @@
       <c r="H69" s="4" t="inlineStr"/>
       <c r="I69" s="4" t="inlineStr"/>
       <c r="J69" s="4" t="inlineStr"/>
-      <c r="K69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L69" s="4" t="inlineStr"/>
     </row>
     <row r="70" ht="18" customHeight="1">
-      <c r="A70" s="2" t="inlineStr"/>
-      <c r="B70" s="2" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+          <t>BC - Resolução BCB N° 577 de 23/06/2026</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -8823,8 +9387,140 @@
       </c>
       <c r="L70" s="2" t="inlineStr"/>
     </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 578 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="2" t="inlineStr"/>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr"/>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr"/>
+      <c r="J73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="2" t="inlineStr"/>
+      <c r="B74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="4" t="inlineStr"/>
+      <c r="B75" s="4" t="inlineStr"/>
+      <c r="C75" s="4" t="inlineStr"/>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="2" t="inlineStr"/>
+      <c r="B76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L70"/>
+  <autoFilter ref="A1:L76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9246,7 +9942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -10537,8 +11233,158 @@
       <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
     </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52940</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 578 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52939</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 577 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52938</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Resolução BCB</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 576 de 23/06/2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L26"/>
+  <autoFilter ref="A1:L29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: atualiza planilha normativos (2026-06-24 18:55)
</commit_message>
<xml_diff>
--- a/planilha/normativos_radar.xlsx
+++ b/planilha/normativos_radar.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoria" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Normativos'!$A$1:$Q$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pilares'!$A$1:$L$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog NÃO APLICÁVEL'!$A$2:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Auditoria'!$A$1:$L$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q87"/>
+  <dimension ref="A1:Q89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -5772,69 +5772,161 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>normativos_52913</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr"/>
-      <c r="C73" s="4" t="inlineStr"/>
-      <c r="D73" s="4" t="inlineStr"/>
+          <t>normativos_52941</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
       <c r="E73" s="4" t="inlineStr"/>
-      <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" s="4" t="inlineStr"/>
-      <c r="J73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 751 de 24/06/2026</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I73" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K73" s="4" t="inlineStr"/>
-      <c r="L73" s="4" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 751 não é diretamente aplicável mas deve ser monitorada pois divulga as rubricas contábeis do padrão contábil das instituições reguladas pelo banco central do brasil – cosif, utilizadas como base de cálculo das contribuições ordinárias, especiais e adicionais d Temas a acompanhar: banco.
+### Avaliação de Risco:
+[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto F</t>
+        </is>
+      </c>
+      <c r="M73" s="4" t="inlineStr">
+        <is>
+          <t>[Impacto Operacional] Score: BAIXO (1/4) | Justificativa: Impacto operacional não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Regulatório] Score: BAIXO (1/4) | Justificativa: Impacto regulatório não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto Financeiro] Score: BAIXO (1/4) | Justificativa: Impacto financeiro não identificado ou mínimo. | Evidências: nenhuma evidência direta
+[Impacto em Clientes] Score: BAIXO (1/4) | Justificativa: Impacto em clientes não identificado. | Evidências: nenhuma evidência direta
+Score consolidado: BAIXO (média ponderada: 1.00/4.0, divisor 4.5)
+Lógica: Score médio ponderado: 1.00/4.0 (divisor 4.5)
+Fórmula: Operacional×1.0 + Regulatório×1.5 + Financeiro×1.0 + Clientes×1.0, dividido por 4.5. Se qualquer pilar=CRÍTICO → mínimo ALTO.</t>
+        </is>
+      </c>
+      <c r="N73" s="4" t="inlineStr">
+        <is>
+          <t>Divulga as rubricas contábeis do Padrão Contábil das Instituições Reguladas pelo Banco Central do Brasil – Cosif, utilizadas como base de cálculo das contribuições ordinárias, especiais e adicionais d</t>
+        </is>
+      </c>
+      <c r="O73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=751</t>
+        </is>
+      </c>
       <c r="P73" s="4" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
-      <c r="Q73" s="4" t="inlineStr"/>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="Q73" s="4" t="inlineStr">
+        <is>
+          <t>ementa</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>normativos_52911</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr"/>
-      <c r="C74" s="2" t="inlineStr"/>
-      <c r="D74" s="2" t="inlineStr"/>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
+          <t>bc_-_instrução_normativa_bcb_n_751_de_24062026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Verificar texto integral</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 751 de 24/06/2026</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
-      <c r="L74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>A IN BCB nº 751 não é diretamente aplicável mas deve ser monitorada pois divulga as rubricas contábeis do padrão contábil das instituições reguladas pelo banco central do brasil – cosif, utilizadas como base de cálculo das contribuições ordinárias, especiais e adicionais d Temas a acompanhar: banco.</t>
+        </is>
+      </c>
       <c r="M74" s="2" t="inlineStr"/>
-      <c r="N74" s="2" t="inlineStr"/>
-      <c r="O74" s="2" t="inlineStr"/>
-      <c r="P74" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-28</t>
-        </is>
-      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Divulga as rubricas contábeis do Padrão Contábil das Instituições Reguladas pelo Banco Central do Brasil – Cosif, utilizadas como base de cálculo das contribuições ordinárias, especiais e adicionais d</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=751](https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=751</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr"/>
       <c r="Q74" s="2" t="inlineStr"/>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>normativos_52912</t>
+          <t>normativos_52913</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr"/>
@@ -5865,7 +5957,7 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>normativos_52909</t>
+          <t>normativos_52911</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
@@ -5873,9 +5965,9 @@
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -5896,7 +5988,7 @@
     <row r="77" ht="18" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>normativos_52908</t>
+          <t>normativos_52912</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr"/>
@@ -5904,9 +5996,9 @@
       <c r="D77" s="4" t="inlineStr"/>
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="3" t="inlineStr">
-        <is>
-          <t>APLICÁVEL</t>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr"/>
@@ -5927,7 +6019,7 @@
     <row r="78" ht="18" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>normativos_52907</t>
+          <t>normativos_52909</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr"/>
@@ -5958,7 +6050,7 @@
     <row r="79" ht="18" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>normativos_52910</t>
+          <t>normativos_52908</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr"/>
@@ -5989,7 +6081,7 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>normativos_52906</t>
+          <t>normativos_52907</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr"/>
@@ -5997,9 +6089,9 @@
       <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -6020,7 +6112,7 @@
     <row r="81" ht="18" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>normativos_52915</t>
+          <t>normativos_52910</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr"/>
@@ -6028,9 +6120,9 @@
       <c r="D81" s="4" t="inlineStr"/>
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr"/>
-      <c r="G81" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr"/>
@@ -6051,29 +6143,21 @@
     <row r="82" ht="18" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>normativos_52916</t>
+          <t>normativos_52906</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr"/>
       <c r="D82" s="2" t="inlineStr"/>
       <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
-      <c r="G82" s="6" t="inlineStr">
-        <is>
-          <t>MONITORAR</t>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
-      <c r="I82" s="7" t="inlineStr">
-        <is>
-          <t>BAIXO</t>
-        </is>
-      </c>
+      <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr"/>
       <c r="L82" s="2" t="inlineStr"/>
@@ -6090,130 +6174,98 @@
     <row r="83" ht="18" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>normativos_52918</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>739</t>
-        </is>
-      </c>
-      <c r="D83" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-29</t>
-        </is>
-      </c>
+          <t>normativos_52915</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr"/>
+      <c r="C83" s="4" t="inlineStr"/>
+      <c r="D83" s="4" t="inlineStr"/>
       <c r="E83" s="4" t="inlineStr"/>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
-        </is>
-      </c>
+      <c r="F83" s="4" t="inlineStr"/>
       <c r="G83" s="9" t="inlineStr">
         <is>
           <t>NÃO APLICÁVEL</t>
         </is>
       </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
+      <c r="H83" s="4" t="inlineStr"/>
       <c r="I83" s="4" t="inlineStr"/>
       <c r="J83" s="4" t="inlineStr"/>
       <c r="K83" s="4" t="inlineStr"/>
       <c r="L83" s="4" t="inlineStr"/>
       <c r="M83" s="4" t="inlineStr"/>
       <c r="N83" s="4" t="inlineStr"/>
-      <c r="O83" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
-        </is>
-      </c>
-      <c r="P83" s="4" t="inlineStr"/>
+      <c r="O83" s="4" t="inlineStr"/>
+      <c r="P83" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q83" s="4" t="inlineStr"/>
     </row>
     <row r="84" ht="18" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>normativos_52931</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Instrução Normativa BCB</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>747</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+          <t>normativos_52916</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
-        </is>
-      </c>
-      <c r="G84" s="9" t="inlineStr">
-        <is>
-          <t>NÃO APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="inlineStr"/>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="7" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr"/>
       <c r="L84" s="2" t="inlineStr"/>
       <c r="M84" s="2" t="inlineStr"/>
       <c r="N84" s="2" t="inlineStr"/>
-      <c r="O84" s="2" t="inlineStr">
-        <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
-        </is>
-      </c>
-      <c r="P84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr"/>
+      <c r="P84" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
       <c r="Q84" s="2" t="inlineStr"/>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>normativos_52933</t>
+          <t>normativos_52918</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Resolução BCB</t>
+          <t>Instrução Normativa BCB</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>739</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 739 de 29/05/2026</t>
         </is>
       </c>
       <c r="G85" s="9" t="inlineStr">
@@ -6234,7 +6286,7 @@
       <c r="N85" s="4" t="inlineStr"/>
       <c r="O85" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=739</t>
         </is>
       </c>
       <c r="P85" s="4" t="inlineStr"/>
@@ -6243,7 +6295,7 @@
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>normativos_52935</t>
+          <t>normativos_52931</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -6253,18 +6305,18 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>749</t>
+          <t>747</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+          <t>BC - Instrução Normativa BCB N° 747 de 17/06/2026</t>
         </is>
       </c>
       <c r="G86" s="9" t="inlineStr">
@@ -6274,7 +6326,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -6285,7 +6337,7 @@
       <c r="N86" s="2" t="inlineStr"/>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=747</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr"/>
@@ -6294,28 +6346,28 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>normativos_52936</t>
+          <t>normativos_52933</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Instrução Normativa BCB</t>
+          <t>Resolução BCB</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>574</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+          <t>BC - Resolução BCB N° 574 de 18/06/2026</t>
         </is>
       </c>
       <c r="G87" s="9" t="inlineStr">
@@ -6325,7 +6377,7 @@
       </c>
       <c r="H87" s="4" t="inlineStr">
         <is>
-          <t>MÉDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="I87" s="4" t="inlineStr"/>
@@ -6336,14 +6388,116 @@
       <c r="N87" s="4" t="inlineStr"/>
       <c r="O87" s="4" t="inlineStr">
         <is>
-          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=750</t>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Resolu%C3%A7%C3%A3o%20BCB&amp;numero=574</t>
         </is>
       </c>
       <c r="P87" s="4" t="inlineStr"/>
       <c r="Q87" s="4" t="inlineStr"/>
     </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52935</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 749 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G88" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=749</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr"/>
+      <c r="Q88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>normativos_52936</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 750 de 19/06/2026</t>
+        </is>
+      </c>
+      <c r="G89" s="9" t="inlineStr">
+        <is>
+          <t>NÃO APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>MÉDIA</t>
+        </is>
+      </c>
+      <c r="I89" s="4" t="inlineStr"/>
+      <c r="J89" s="4" t="inlineStr"/>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+      <c r="M89" s="4" t="inlineStr"/>
+      <c r="N89" s="4" t="inlineStr"/>
+      <c r="O89" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcb.gov.br/estabilidadefinanceira/exibenormativo?tipo=Instru%C3%A7%C3%A3o%20Normativa%20BCB&amp;numero=750</t>
+        </is>
+      </c>
+      <c r="P89" s="4" t="inlineStr"/>
+      <c r="Q89" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q87"/>
+  <autoFilter ref="A1:Q89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6416,7 +6570,7 @@
       </c>
       <c r="C3" s="12" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -6435,11 +6589,11 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>57%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -6462,7 +6616,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -6481,7 +6635,7 @@
         </is>
       </c>
       <c r="F6" s="13" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7"/>
@@ -6576,7 +6730,7 @@
         </is>
       </c>
       <c r="G13" s="12" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14">
@@ -6586,13 +6740,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>2</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
@@ -6668,7 +6822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -9422,30 +9576,68 @@
       <c r="L71" s="4" t="inlineStr"/>
     </row>
     <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="2" t="inlineStr"/>
-      <c r="B72" s="2" t="inlineStr"/>
-      <c r="C72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 751 de 24/06/2026</t>
+        </is>
+      </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr"/>
-      <c r="K72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L72" s="2" t="inlineStr"/>
     </row>
     <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="4" t="inlineStr"/>
-      <c r="B73" s="4" t="inlineStr"/>
-      <c r="C73" s="4" t="inlineStr"/>
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 751 de 24/06/2026</t>
+        </is>
+      </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>APLICÁVEL</t>
+          <t>MONITORAR</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr"/>
@@ -9454,7 +9646,11 @@
       <c r="H73" s="4" t="inlineStr"/>
       <c r="I73" s="4" t="inlineStr"/>
       <c r="J73" s="4" t="inlineStr"/>
-      <c r="K73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
       <c r="L73" s="4" t="inlineStr"/>
     </row>
     <row r="74" ht="18" customHeight="1">
@@ -9496,14 +9692,10 @@
     <row r="76" ht="18" customHeight="1">
       <c r="A76" s="2" t="inlineStr"/>
       <c r="B76" s="2" t="inlineStr"/>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
-        </is>
-      </c>
+      <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>MONITORAR</t>
+          <t>APLICÁVEL</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
@@ -9512,15 +9704,55 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="inlineStr"/>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="4" t="inlineStr"/>
+      <c r="B77" s="4" t="inlineStr"/>
+      <c r="C77" s="4" t="inlineStr"/>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>APLICÁVEL</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr"/>
+      <c r="H77" s="4" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr"/>
+      <c r="J77" s="4" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="2" t="inlineStr"/>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>BC - Resolução BCB N° 571 de 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
         <is>
           <t>BAIXO</t>
         </is>
       </c>
-      <c r="L76" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L76"/>
+  <autoFilter ref="A1:L78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9942,7 +10174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -11383,8 +11615,58 @@
       <c r="K29" s="4" t="inlineStr"/>
       <c r="L29" s="4" t="inlineStr"/>
     </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>normativos_52941</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Instrução Normativa BCB</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>751</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>BC - Instrução Normativa BCB N° 751 de 24/06/2026</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>MONITORAR</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>inicial</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>BAIXO</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:L30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>